<commit_message>
workday clean up, code runs the same, bunch of stuff deleted and compacted
code runs the same
</commit_message>
<xml_diff>
--- a/SizingParams.xlsx
+++ b/SizingParams.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\Desktop\Fall 2026\AAE 451\451-DBF-Team01\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ceaa8977d2236823/Documents/GitHub/451-DBF-Team01/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8FE2283-5D42-44E7-810A-D88494F7A345}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="77" documentId="13_ncr:1_{B8FE2283-5D42-44E7-810A-D88494F7A345}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CFC54096-9E1B-46ED-AC3C-8C70B6949F5A}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5136" yWindow="1980" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INPUTS" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="234">
   <si>
     <t>Parameter</t>
   </si>
@@ -685,6 +685,78 @@
   </si>
   <si>
     <t>Parasitic drag</t>
+  </si>
+  <si>
+    <t>CM_0_Wing</t>
+  </si>
+  <si>
+    <t>CM of Wing at 0 AoA</t>
+  </si>
+  <si>
+    <t>Airfoil_Alpha_Stall</t>
+  </si>
+  <si>
+    <t>kappa</t>
+  </si>
+  <si>
+    <t>AR_v</t>
+  </si>
+  <si>
+    <t>Vertical Tail Aspect Ratio</t>
+  </si>
+  <si>
+    <t>E_r</t>
+  </si>
+  <si>
+    <t>Rudder Chord Fraction</t>
+  </si>
+  <si>
+    <t>delta_r_limit</t>
+  </si>
+  <si>
+    <t>Max Rudder Deflection</t>
+  </si>
+  <si>
+    <t>crosswind_ratio</t>
+  </si>
+  <si>
+    <t>Cross Wind Ratio</t>
+  </si>
+  <si>
+    <t>roll_rate_target_dps</t>
+  </si>
+  <si>
+    <t>deg/s</t>
+  </si>
+  <si>
+    <t>Roll Rate Target</t>
+  </si>
+  <si>
+    <t>E_a</t>
+  </si>
+  <si>
+    <t>Aileron Chord Fraction</t>
+  </si>
+  <si>
+    <t>y1_frac</t>
+  </si>
+  <si>
+    <t>y2_frac</t>
+  </si>
+  <si>
+    <t>Aileron Span Fractions of the Semi Span</t>
+  </si>
+  <si>
+    <t>delta_a_limit</t>
+  </si>
+  <si>
+    <t>Max Aileron Deflection</t>
+  </si>
+  <si>
+    <t>Gamma_dihedral_deg</t>
+  </si>
+  <si>
+    <t>Dihedral Initialization</t>
   </si>
 </sst>
 </file>
@@ -731,7 +803,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -862,11 +934,46 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="10"/>
+      </left>
+      <right style="thin">
+        <color indexed="10"/>
+      </right>
+      <top style="thin">
+        <color indexed="10"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="10"/>
+      </left>
+      <right style="thin">
+        <color indexed="10"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="10"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="10"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
@@ -901,6 +1008,14 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1089,15 +1204,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>142142</xdr:colOff>
-      <xdr:row>83</xdr:row>
-      <xdr:rowOff>97457</xdr:rowOff>
+      <xdr:colOff>179294</xdr:colOff>
+      <xdr:row>120</xdr:row>
+      <xdr:rowOff>167247</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>605269</xdr:colOff>
-      <xdr:row>100</xdr:row>
-      <xdr:rowOff>59358</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1096331</xdr:colOff>
+      <xdr:row>132</xdr:row>
+      <xdr:rowOff>166935</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1120,8 +1235,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="142142" y="14937407"/>
-          <a:ext cx="5206577" cy="3038476"/>
+          <a:off x="179294" y="21682541"/>
+          <a:ext cx="4718072" cy="2151218"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1236,15 +1351,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>175846</xdr:colOff>
-      <xdr:row>96</xdr:row>
-      <xdr:rowOff>43014</xdr:rowOff>
+      <xdr:colOff>212997</xdr:colOff>
+      <xdr:row>128</xdr:row>
+      <xdr:rowOff>150591</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>575716</xdr:colOff>
-      <xdr:row>104</xdr:row>
-      <xdr:rowOff>65005</xdr:rowOff>
+      <xdr:colOff>612867</xdr:colOff>
+      <xdr:row>136</xdr:row>
+      <xdr:rowOff>172582</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1267,8 +1382,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="175846" y="17261283"/>
-          <a:ext cx="4920582" cy="1487376"/>
+          <a:off x="212997" y="23100238"/>
+          <a:ext cx="8073658" cy="1456344"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1285,15 +1400,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>278424</xdr:colOff>
-      <xdr:row>104</xdr:row>
-      <xdr:rowOff>14660</xdr:rowOff>
+      <xdr:colOff>296354</xdr:colOff>
+      <xdr:row>117</xdr:row>
+      <xdr:rowOff>23624</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>1516674</xdr:colOff>
-      <xdr:row>106</xdr:row>
-      <xdr:rowOff>118773</xdr:rowOff>
+      <xdr:colOff>1534604</xdr:colOff>
+      <xdr:row>119</xdr:row>
+      <xdr:rowOff>127737</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1316,8 +1431,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="278424" y="18698314"/>
-          <a:ext cx="5758962" cy="470459"/>
+          <a:off x="296354" y="21001036"/>
+          <a:ext cx="8912038" cy="462701"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1383,15 +1498,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>498231</xdr:colOff>
-      <xdr:row>106</xdr:row>
-      <xdr:rowOff>109907</xdr:rowOff>
+      <xdr:colOff>535382</xdr:colOff>
+      <xdr:row>139</xdr:row>
+      <xdr:rowOff>38190</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>1281404</xdr:colOff>
-      <xdr:row>122</xdr:row>
-      <xdr:rowOff>79550</xdr:rowOff>
+      <xdr:colOff>1318555</xdr:colOff>
+      <xdr:row>155</xdr:row>
+      <xdr:rowOff>7833</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1414,8 +1529,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="498231" y="19159907"/>
-          <a:ext cx="5062096" cy="2900412"/>
+          <a:off x="535382" y="24960072"/>
+          <a:ext cx="8456961" cy="2838349"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1432,15 +1547,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>685067</xdr:colOff>
-      <xdr:row>124</xdr:row>
-      <xdr:rowOff>52020</xdr:rowOff>
+      <xdr:colOff>722218</xdr:colOff>
+      <xdr:row>156</xdr:row>
+      <xdr:rowOff>159598</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>1305657</xdr:colOff>
-      <xdr:row>139</xdr:row>
-      <xdr:rowOff>59792</xdr:rowOff>
+      <xdr:colOff>1342808</xdr:colOff>
+      <xdr:row>171</xdr:row>
+      <xdr:rowOff>167369</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1463,8 +1578,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="685067" y="22399135"/>
-          <a:ext cx="4899513" cy="2755369"/>
+          <a:off x="722218" y="28129480"/>
+          <a:ext cx="8294378" cy="2697183"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2620,21 +2735,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S132"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.85" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.85" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.42578125" style="32" customWidth="1"/>
-    <col min="3" max="3" width="9.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.7109375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="34.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.7109375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="40.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="20" width="8.7109375" style="1" customWidth="1"/>
-    <col min="21" max="16384" width="8.7109375" style="1"/>
+    <col min="1" max="1" width="18.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.44140625" style="32" customWidth="1"/>
+    <col min="3" max="3" width="9.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.6640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="34.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.6640625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="40.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="20" width="8.6640625" style="1" customWidth="1"/>
+    <col min="21" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
@@ -2671,7 +2786,7 @@
       <c r="R1" s="3"/>
       <c r="S1" s="3"/>
     </row>
-    <row r="2" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="11" t="s">
         <v>5</v>
       </c>
@@ -2706,7 +2821,7 @@
       <c r="R2" s="3"/>
       <c r="S2" s="3"/>
     </row>
-    <row r="3" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
         <v>10</v>
       </c>
@@ -2739,7 +2854,7 @@
       <c r="R3" s="3"/>
       <c r="S3" s="3"/>
     </row>
-    <row r="4" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
         <v>14</v>
       </c>
@@ -2772,7 +2887,7 @@
       <c r="R4" s="3"/>
       <c r="S4" s="3"/>
     </row>
-    <row r="5" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
         <v>17</v>
       </c>
@@ -2807,7 +2922,7 @@
       <c r="R5" s="3"/>
       <c r="S5" s="3"/>
     </row>
-    <row r="6" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
         <v>22</v>
       </c>
@@ -2842,7 +2957,7 @@
       <c r="R6" s="3"/>
       <c r="S6" s="3"/>
     </row>
-    <row r="7" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="12" t="s">
         <v>178</v>
       </c>
@@ -2876,7 +2991,7 @@
       <c r="R7" s="3"/>
       <c r="S7" s="3"/>
     </row>
-    <row r="8" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>26</v>
       </c>
@@ -2912,7 +3027,7 @@
       <c r="R8" s="3"/>
       <c r="S8" s="3"/>
     </row>
-    <row r="9" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="12" t="s">
         <v>183</v>
       </c>
@@ -2946,7 +3061,7 @@
       <c r="R9" s="3"/>
       <c r="S9" s="3"/>
     </row>
-    <row r="10" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
         <v>32</v>
       </c>
@@ -2982,7 +3097,7 @@
       <c r="R10" s="3"/>
       <c r="S10" s="3"/>
     </row>
-    <row r="11" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
         <v>35</v>
       </c>
@@ -3017,7 +3132,7 @@
       <c r="R11" s="3"/>
       <c r="S11" s="3"/>
     </row>
-    <row r="12" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
         <v>39</v>
       </c>
@@ -3053,7 +3168,7 @@
       <c r="R12" s="3"/>
       <c r="S12" s="3"/>
     </row>
-    <row r="13" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="11" t="s">
         <v>43</v>
       </c>
@@ -3089,7 +3204,7 @@
       <c r="R13" s="3"/>
       <c r="S13" s="3"/>
     </row>
-    <row r="14" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
         <v>47</v>
       </c>
@@ -3126,7 +3241,7 @@
       <c r="R14" s="3"/>
       <c r="S14" s="3"/>
     </row>
-    <row r="15" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="12" t="s">
         <v>141</v>
       </c>
@@ -3160,7 +3275,7 @@
       <c r="R15" s="3"/>
       <c r="S15" s="3"/>
     </row>
-    <row r="16" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
         <v>52</v>
       </c>
@@ -3196,7 +3311,7 @@
       <c r="R16" s="3"/>
       <c r="S16" s="3"/>
     </row>
-    <row r="17" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
         <v>55</v>
       </c>
@@ -3230,7 +3345,7 @@
       <c r="R17" s="3"/>
       <c r="S17" s="3"/>
     </row>
-    <row r="18" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
         <v>58</v>
       </c>
@@ -3264,7 +3379,7 @@
       <c r="R18" s="3"/>
       <c r="S18" s="3"/>
     </row>
-    <row r="19" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="11" t="s">
         <v>61</v>
       </c>
@@ -3297,7 +3412,7 @@
       <c r="R19" s="3"/>
       <c r="S19" s="3"/>
     </row>
-    <row r="20" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="11" t="s">
         <v>64</v>
       </c>
@@ -3330,7 +3445,7 @@
       <c r="R20" s="3"/>
       <c r="S20" s="3"/>
     </row>
-    <row r="21" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="11" t="s">
         <v>66</v>
       </c>
@@ -3364,7 +3479,7 @@
       <c r="R21" s="3"/>
       <c r="S21" s="3"/>
     </row>
-    <row r="22" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="11" t="s">
         <v>68</v>
       </c>
@@ -3397,7 +3512,7 @@
       <c r="R22" s="3"/>
       <c r="S22" s="3"/>
     </row>
-    <row r="23" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="11" t="s">
         <v>71</v>
       </c>
@@ -3429,7 +3544,7 @@
       <c r="R23" s="3"/>
       <c r="S23" s="3"/>
     </row>
-    <row r="24" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="11" t="s">
         <v>73</v>
       </c>
@@ -3463,7 +3578,7 @@
       <c r="R24" s="3"/>
       <c r="S24" s="3"/>
     </row>
-    <row r="25" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="11" t="s">
         <v>76</v>
       </c>
@@ -3496,7 +3611,7 @@
       <c r="R25" s="3"/>
       <c r="S25" s="3"/>
     </row>
-    <row r="26" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="11" t="s">
         <v>79</v>
       </c>
@@ -3529,7 +3644,7 @@
       <c r="R26" s="3"/>
       <c r="S26" s="3"/>
     </row>
-    <row r="27" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="11" t="s">
         <v>82</v>
       </c>
@@ -3561,7 +3676,7 @@
       <c r="R27" s="3"/>
       <c r="S27" s="3"/>
     </row>
-    <row r="28" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="11" t="s">
         <v>85</v>
       </c>
@@ -3594,7 +3709,7 @@
       <c r="R28" s="3"/>
       <c r="S28" s="3"/>
     </row>
-    <row r="29" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="11" t="s">
         <v>88</v>
       </c>
@@ -3627,7 +3742,7 @@
       <c r="R29" s="3"/>
       <c r="S29" s="3"/>
     </row>
-    <row r="30" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="11" t="s">
         <v>91</v>
       </c>
@@ -3660,7 +3775,7 @@
       <c r="R30" s="3"/>
       <c r="S30" s="3"/>
     </row>
-    <row r="31" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="11" t="s">
         <v>93</v>
       </c>
@@ -3693,7 +3808,7 @@
       <c r="R31" s="3"/>
       <c r="S31" s="3"/>
     </row>
-    <row r="32" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="11" t="s">
         <v>96</v>
       </c>
@@ -3726,7 +3841,7 @@
       <c r="R32" s="3"/>
       <c r="S32" s="3"/>
     </row>
-    <row r="33" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="11" t="s">
         <v>99</v>
       </c>
@@ -3758,7 +3873,7 @@
       <c r="R33" s="3"/>
       <c r="S33" s="3"/>
     </row>
-    <row r="34" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="11" t="s">
         <v>101</v>
       </c>
@@ -3791,7 +3906,7 @@
       <c r="R34" s="3"/>
       <c r="S34" s="3"/>
     </row>
-    <row r="35" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="11" t="s">
         <v>104</v>
       </c>
@@ -3822,7 +3937,7 @@
       <c r="R35" s="3"/>
       <c r="S35" s="3"/>
     </row>
-    <row r="36" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="11" t="s">
         <v>107</v>
       </c>
@@ -3853,7 +3968,7 @@
       <c r="R36" s="3"/>
       <c r="S36" s="3"/>
     </row>
-    <row r="37" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="11" t="s">
         <v>110</v>
       </c>
@@ -3884,7 +3999,7 @@
       <c r="R37" s="3"/>
       <c r="S37" s="3"/>
     </row>
-    <row r="38" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="11" t="s">
         <v>112</v>
       </c>
@@ -3917,7 +4032,7 @@
       <c r="R38" s="3"/>
       <c r="S38" s="3"/>
     </row>
-    <row r="39" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="11" t="s">
         <v>116</v>
       </c>
@@ -3949,7 +4064,7 @@
       <c r="R39" s="3"/>
       <c r="S39" s="3"/>
     </row>
-    <row r="40" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="11" t="s">
         <v>119</v>
       </c>
@@ -3981,7 +4096,7 @@
       <c r="R40" s="3"/>
       <c r="S40" s="3"/>
     </row>
-    <row r="41" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="12" t="s">
         <v>142</v>
       </c>
@@ -4014,7 +4129,7 @@
       <c r="R41" s="3"/>
       <c r="S41" s="3"/>
     </row>
-    <row r="42" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="12" t="s">
         <v>180</v>
       </c>
@@ -4044,7 +4159,7 @@
       <c r="R42" s="3"/>
       <c r="S42" s="3"/>
     </row>
-    <row r="43" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="11" t="s">
         <v>125</v>
       </c>
@@ -4075,7 +4190,7 @@
       <c r="R43" s="3"/>
       <c r="S43" s="3"/>
     </row>
-    <row r="44" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="12" t="s">
         <v>127</v>
       </c>
@@ -4106,7 +4221,7 @@
       <c r="R44" s="3"/>
       <c r="S44" s="3"/>
     </row>
-    <row r="45" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="12" t="s">
         <v>189</v>
       </c>
@@ -4137,7 +4252,7 @@
       <c r="R45" s="3"/>
       <c r="S45" s="3"/>
     </row>
-    <row r="46" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="11" t="s">
         <v>130</v>
       </c>
@@ -4170,7 +4285,7 @@
       <c r="R46" s="3"/>
       <c r="S46" s="3"/>
     </row>
-    <row r="47" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="11" t="s">
         <v>133</v>
       </c>
@@ -4203,7 +4318,7 @@
       <c r="R47" s="3"/>
       <c r="S47" s="3"/>
     </row>
-    <row r="48" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="12" t="s">
         <v>158</v>
       </c>
@@ -4236,7 +4351,7 @@
       <c r="R48" s="3"/>
       <c r="S48" s="3"/>
     </row>
-    <row r="49" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="12" t="s">
         <v>157</v>
       </c>
@@ -4265,7 +4380,7 @@
       <c r="R49" s="3"/>
       <c r="S49" s="3"/>
     </row>
-    <row r="50" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="12" t="s">
         <v>164</v>
       </c>
@@ -4299,7 +4414,7 @@
       <c r="R50" s="3"/>
       <c r="S50" s="3"/>
     </row>
-    <row r="51" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="13" t="s">
         <v>139</v>
       </c>
@@ -4332,7 +4447,7 @@
       <c r="R51" s="3"/>
       <c r="S51" s="3"/>
     </row>
-    <row r="52" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="13" t="s">
         <v>186</v>
       </c>
@@ -4364,7 +4479,7 @@
       <c r="R52" s="3"/>
       <c r="S52" s="3"/>
     </row>
-    <row r="53" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="14" t="s">
         <v>143</v>
       </c>
@@ -4395,7 +4510,7 @@
       <c r="R53" s="3"/>
       <c r="S53" s="3"/>
     </row>
-    <row r="54" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="13" t="s">
         <v>147</v>
       </c>
@@ -4426,7 +4541,7 @@
       <c r="R54" s="3"/>
       <c r="S54" s="3"/>
     </row>
-    <row r="55" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="13" t="s">
         <v>149</v>
       </c>
@@ -4457,7 +4572,7 @@
       <c r="R55" s="3"/>
       <c r="S55" s="3"/>
     </row>
-    <row r="56" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="13" t="s">
         <v>148</v>
       </c>
@@ -4488,7 +4603,7 @@
       <c r="R56" s="3"/>
       <c r="S56" s="3"/>
     </row>
-    <row r="57" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="13" t="s">
         <v>151</v>
       </c>
@@ -4519,7 +4634,7 @@
       <c r="R57" s="3"/>
       <c r="S57" s="3"/>
     </row>
-    <row r="58" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="13" t="s">
         <v>160</v>
       </c>
@@ -4550,7 +4665,7 @@
       <c r="R58" s="3"/>
       <c r="S58" s="3"/>
     </row>
-    <row r="59" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="13" t="s">
         <v>155</v>
       </c>
@@ -4581,7 +4696,7 @@
       <c r="R59" s="3"/>
       <c r="S59" s="3"/>
     </row>
-    <row r="60" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="13" t="s">
         <v>159</v>
       </c>
@@ -4612,7 +4727,7 @@
       <c r="R60" s="3"/>
       <c r="S60" s="3"/>
     </row>
-    <row r="61" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="13" t="s">
         <v>161</v>
       </c>
@@ -4643,7 +4758,7 @@
       <c r="R61" s="3"/>
       <c r="S61" s="3"/>
     </row>
-    <row r="62" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="13" t="s">
         <v>162</v>
       </c>
@@ -4672,7 +4787,7 @@
       <c r="R62" s="3"/>
       <c r="S62" s="3"/>
     </row>
-    <row r="63" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="13" t="s">
         <v>163</v>
       </c>
@@ -4701,7 +4816,7 @@
       <c r="R63" s="3"/>
       <c r="S63" s="3"/>
     </row>
-    <row r="64" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="13" t="s">
         <v>165</v>
       </c>
@@ -4731,7 +4846,7 @@
       <c r="R64" s="3"/>
       <c r="S64" s="3"/>
     </row>
-    <row r="65" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="13" t="s">
         <v>181</v>
       </c>
@@ -4762,7 +4877,7 @@
       <c r="R65" s="3"/>
       <c r="S65" s="3"/>
     </row>
-    <row r="66" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="13" t="s">
         <v>182</v>
       </c>
@@ -4793,7 +4908,7 @@
       <c r="R66" s="3"/>
       <c r="S66" s="3"/>
     </row>
-    <row r="67" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="13" t="s">
         <v>166</v>
       </c>
@@ -4822,7 +4937,7 @@
       <c r="R67" s="3"/>
       <c r="S67" s="3"/>
     </row>
-    <row r="68" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="13" t="s">
         <v>167</v>
       </c>
@@ -4851,7 +4966,7 @@
       <c r="R68" s="3"/>
       <c r="S68" s="3"/>
     </row>
-    <row r="69" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="13" t="s">
         <v>168</v>
       </c>
@@ -4880,7 +4995,7 @@
       <c r="R69" s="3"/>
       <c r="S69" s="3"/>
     </row>
-    <row r="70" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="13" t="s">
         <v>169</v>
       </c>
@@ -4909,7 +5024,7 @@
       <c r="R70" s="3"/>
       <c r="S70" s="3"/>
     </row>
-    <row r="71" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="13" t="s">
         <v>170</v>
       </c>
@@ -4938,7 +5053,7 @@
       <c r="R71" s="3"/>
       <c r="S71" s="3"/>
     </row>
-    <row r="72" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="13" t="s">
         <v>171</v>
       </c>
@@ -4967,7 +5082,7 @@
       <c r="R72" s="3"/>
       <c r="S72" s="3"/>
     </row>
-    <row r="73" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="13" t="s">
         <v>172</v>
       </c>
@@ -4996,7 +5111,7 @@
       <c r="R73" s="3"/>
       <c r="S73" s="3"/>
     </row>
-    <row r="74" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="13" t="s">
         <v>173</v>
       </c>
@@ -5025,7 +5140,7 @@
       <c r="R74" s="3"/>
       <c r="S74" s="3"/>
     </row>
-    <row r="75" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="13" t="s">
         <v>174</v>
       </c>
@@ -5056,7 +5171,7 @@
       <c r="R75" s="3"/>
       <c r="S75" s="3"/>
     </row>
-    <row r="76" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="13" t="s">
         <v>176</v>
       </c>
@@ -5087,7 +5202,7 @@
       <c r="R76" s="3"/>
       <c r="S76" s="3"/>
     </row>
-    <row r="77" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="13" t="s">
         <v>192</v>
       </c>
@@ -5116,7 +5231,7 @@
       <c r="R77" s="3"/>
       <c r="S77" s="3"/>
     </row>
-    <row r="78" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="14" t="s">
         <v>193</v>
       </c>
@@ -5147,7 +5262,7 @@
       <c r="R78" s="3"/>
       <c r="S78" s="3"/>
     </row>
-    <row r="79" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="14" t="s">
         <v>196</v>
       </c>
@@ -5178,7 +5293,7 @@
       <c r="R79" s="3"/>
       <c r="S79" s="3"/>
     </row>
-    <row r="80" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="14" t="s">
         <v>197</v>
       </c>
@@ -5209,12 +5324,22 @@
       <c r="R80" s="3"/>
       <c r="S80" s="3"/>
     </row>
-    <row r="81" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="14"/>
-      <c r="B81" s="31"/>
-      <c r="C81" s="28"/>
-      <c r="D81" s="3"/>
-      <c r="E81" s="3"/>
+    <row r="81" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="14" t="s">
+        <v>210</v>
+      </c>
+      <c r="B81" s="31" t="s">
+        <v>204</v>
+      </c>
+      <c r="C81" s="28">
+        <v>-0.08</v>
+      </c>
+      <c r="D81" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="E81" s="3" t="s">
+        <v>211</v>
+      </c>
       <c r="F81" s="3"/>
       <c r="G81" s="3"/>
       <c r="H81" s="3"/>
@@ -5230,11 +5355,19 @@
       <c r="R81" s="3"/>
       <c r="S81" s="3"/>
     </row>
-    <row r="82" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="14"/>
-      <c r="B82" s="31"/>
-      <c r="C82" s="28"/>
-      <c r="D82" s="3"/>
+    <row r="82" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A82" s="14" t="s">
+        <v>212</v>
+      </c>
+      <c r="B82" s="31" t="s">
+        <v>204</v>
+      </c>
+      <c r="C82" s="28">
+        <v>15.8</v>
+      </c>
+      <c r="D82" s="3" t="s">
+        <v>83</v>
+      </c>
       <c r="E82" s="3"/>
       <c r="F82" s="3"/>
       <c r="G82" s="3"/>
@@ -5251,11 +5384,19 @@
       <c r="R82" s="3"/>
       <c r="S82" s="3"/>
     </row>
-    <row r="83" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="14"/>
-      <c r="B83" s="31"/>
-      <c r="C83" s="28"/>
-      <c r="D83" s="3"/>
+    <row r="83" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="14" t="s">
+        <v>213</v>
+      </c>
+      <c r="B83" s="31" t="s">
+        <v>205</v>
+      </c>
+      <c r="C83" s="28">
+        <v>2</v>
+      </c>
+      <c r="D83" s="9" t="s">
+        <v>194</v>
+      </c>
       <c r="E83" s="3"/>
       <c r="F83" s="3"/>
       <c r="G83" s="3"/>
@@ -5272,12 +5413,22 @@
       <c r="R83" s="3"/>
       <c r="S83" s="3"/>
     </row>
-    <row r="84" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="14"/>
-      <c r="B84" s="31"/>
-      <c r="C84" s="28"/>
-      <c r="D84" s="3"/>
-      <c r="E84" s="3"/>
+    <row r="84" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A84" s="14" t="s">
+        <v>214</v>
+      </c>
+      <c r="B84" s="31" t="s">
+        <v>205</v>
+      </c>
+      <c r="C84" s="28">
+        <v>1.5</v>
+      </c>
+      <c r="D84" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="E84" s="3" t="s">
+        <v>215</v>
+      </c>
       <c r="F84" s="3"/>
       <c r="G84" s="3"/>
       <c r="H84" s="3"/>
@@ -5293,12 +5444,22 @@
       <c r="R84" s="3"/>
       <c r="S84" s="3"/>
     </row>
-    <row r="85" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="14"/>
-      <c r="B85" s="31"/>
-      <c r="C85" s="28"/>
-      <c r="D85" s="3"/>
-      <c r="E85" s="3"/>
+    <row r="85" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A85" s="14" t="s">
+        <v>216</v>
+      </c>
+      <c r="B85" s="31" t="s">
+        <v>205</v>
+      </c>
+      <c r="C85" s="28">
+        <v>0.3</v>
+      </c>
+      <c r="D85" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="E85" s="3" t="s">
+        <v>217</v>
+      </c>
       <c r="F85" s="3"/>
       <c r="G85" s="3"/>
       <c r="H85" s="3"/>
@@ -5314,12 +5475,22 @@
       <c r="R85" s="3"/>
       <c r="S85" s="3"/>
     </row>
-    <row r="86" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="14"/>
-      <c r="B86" s="31"/>
-      <c r="C86" s="28"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="3"/>
+    <row r="86" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A86" s="14" t="s">
+        <v>218</v>
+      </c>
+      <c r="B86" s="31" t="s">
+        <v>205</v>
+      </c>
+      <c r="C86" s="28">
+        <v>20</v>
+      </c>
+      <c r="D86" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E86" s="3" t="s">
+        <v>219</v>
+      </c>
       <c r="F86" s="3"/>
       <c r="G86" s="3"/>
       <c r="H86" s="3"/>
@@ -5335,12 +5506,22 @@
       <c r="R86" s="3"/>
       <c r="S86" s="3"/>
     </row>
-    <row r="87" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="14"/>
-      <c r="B87" s="31"/>
-      <c r="C87" s="28"/>
-      <c r="D87" s="3"/>
-      <c r="E87" s="3"/>
+    <row r="87" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="14" t="s">
+        <v>220</v>
+      </c>
+      <c r="B87" s="31" t="s">
+        <v>204</v>
+      </c>
+      <c r="C87" s="28">
+        <v>0.2</v>
+      </c>
+      <c r="D87" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="E87" s="3" t="s">
+        <v>221</v>
+      </c>
       <c r="F87" s="3"/>
       <c r="G87" s="3"/>
       <c r="H87" s="3"/>
@@ -5356,12 +5537,22 @@
       <c r="R87" s="3"/>
       <c r="S87" s="3"/>
     </row>
-    <row r="88" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="14"/>
-      <c r="B88" s="31"/>
-      <c r="C88" s="28"/>
-      <c r="D88" s="3"/>
-      <c r="E88" s="3"/>
+    <row r="88" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A88" s="14" t="s">
+        <v>222</v>
+      </c>
+      <c r="B88" s="32" t="s">
+        <v>204</v>
+      </c>
+      <c r="C88" s="31">
+        <v>120</v>
+      </c>
+      <c r="D88" s="28" t="s">
+        <v>223</v>
+      </c>
+      <c r="E88" s="3" t="s">
+        <v>224</v>
+      </c>
       <c r="F88" s="3"/>
       <c r="G88" s="3"/>
       <c r="H88" s="3"/>
@@ -5377,12 +5568,22 @@
       <c r="R88" s="3"/>
       <c r="S88" s="3"/>
     </row>
-    <row r="89" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A89" s="14"/>
-      <c r="B89" s="31"/>
-      <c r="C89" s="28"/>
-      <c r="D89" s="3"/>
-      <c r="E89" s="3"/>
+    <row r="89" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A89" s="13" t="s">
+        <v>225</v>
+      </c>
+      <c r="B89" s="34" t="s">
+        <v>205</v>
+      </c>
+      <c r="C89" s="28">
+        <v>0.25</v>
+      </c>
+      <c r="D89" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="E89" s="6" t="s">
+        <v>226</v>
+      </c>
       <c r="F89" s="3"/>
       <c r="G89" s="3"/>
       <c r="H89" s="3"/>
@@ -5398,12 +5599,22 @@
       <c r="R89" s="3"/>
       <c r="S89" s="3"/>
     </row>
-    <row r="90" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A90" s="14"/>
-      <c r="B90" s="31"/>
-      <c r="C90" s="28"/>
-      <c r="D90" s="3"/>
-      <c r="E90" s="3"/>
+    <row r="90" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A90" s="13" t="s">
+        <v>227</v>
+      </c>
+      <c r="B90" s="34" t="s">
+        <v>205</v>
+      </c>
+      <c r="C90" s="28">
+        <v>0.7</v>
+      </c>
+      <c r="D90" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="E90" s="36" t="s">
+        <v>229</v>
+      </c>
       <c r="F90" s="3"/>
       <c r="G90" s="3"/>
       <c r="H90" s="3"/>
@@ -5419,12 +5630,20 @@
       <c r="R90" s="3"/>
       <c r="S90" s="3"/>
     </row>
-    <row r="91" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="14"/>
-      <c r="B91" s="31"/>
-      <c r="C91" s="28"/>
-      <c r="D91" s="3"/>
-      <c r="E91" s="3"/>
+    <row r="91" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A91" s="13" t="s">
+        <v>228</v>
+      </c>
+      <c r="B91" s="34" t="s">
+        <v>205</v>
+      </c>
+      <c r="C91" s="28">
+        <v>1</v>
+      </c>
+      <c r="D91" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="E91" s="37"/>
       <c r="F91" s="3"/>
       <c r="G91" s="3"/>
       <c r="H91" s="3"/>
@@ -5440,12 +5659,22 @@
       <c r="R91" s="3"/>
       <c r="S91" s="3"/>
     </row>
-    <row r="92" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A92" s="14"/>
-      <c r="B92" s="31"/>
-      <c r="C92" s="28"/>
-      <c r="D92" s="3"/>
-      <c r="E92" s="3"/>
+    <row r="92" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A92" s="14" t="s">
+        <v>230</v>
+      </c>
+      <c r="B92" s="31" t="s">
+        <v>205</v>
+      </c>
+      <c r="C92" s="28">
+        <v>15</v>
+      </c>
+      <c r="D92" s="35" t="s">
+        <v>83</v>
+      </c>
+      <c r="E92" s="3" t="s">
+        <v>231</v>
+      </c>
       <c r="F92" s="3"/>
       <c r="G92" s="3"/>
       <c r="H92" s="3"/>
@@ -5461,12 +5690,22 @@
       <c r="R92" s="3"/>
       <c r="S92" s="3"/>
     </row>
-    <row r="93" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="14"/>
-      <c r="B93" s="31"/>
-      <c r="C93" s="28"/>
-      <c r="D93" s="3"/>
-      <c r="E93" s="3"/>
+    <row r="93" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A93" s="14" t="s">
+        <v>232</v>
+      </c>
+      <c r="B93" s="31" t="s">
+        <v>205</v>
+      </c>
+      <c r="C93" s="28">
+        <v>4</v>
+      </c>
+      <c r="D93" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E93" s="3" t="s">
+        <v>233</v>
+      </c>
       <c r="F93" s="3"/>
       <c r="G93" s="3"/>
       <c r="H93" s="3"/>
@@ -5482,7 +5721,7 @@
       <c r="R93" s="3"/>
       <c r="S93" s="3"/>
     </row>
-    <row r="94" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="14"/>
       <c r="B94" s="31"/>
       <c r="C94" s="28"/>
@@ -5503,7 +5742,7 @@
       <c r="R94" s="3"/>
       <c r="S94" s="3"/>
     </row>
-    <row r="95" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="14"/>
       <c r="B95" s="31"/>
       <c r="C95" s="28"/>
@@ -5524,7 +5763,7 @@
       <c r="R95" s="3"/>
       <c r="S95" s="3"/>
     </row>
-    <row r="96" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="14"/>
       <c r="B96" s="31"/>
       <c r="C96" s="28"/>
@@ -5545,7 +5784,7 @@
       <c r="R96" s="3"/>
       <c r="S96" s="3"/>
     </row>
-    <row r="97" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="14"/>
       <c r="B97" s="31"/>
       <c r="C97" s="28"/>
@@ -5566,7 +5805,7 @@
       <c r="R97" s="3"/>
       <c r="S97" s="3"/>
     </row>
-    <row r="98" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="14"/>
       <c r="B98" s="31"/>
       <c r="C98" s="28"/>
@@ -5587,7 +5826,7 @@
       <c r="R98" s="3"/>
       <c r="S98" s="3"/>
     </row>
-    <row r="99" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="14"/>
       <c r="B99" s="31"/>
       <c r="C99" s="28"/>
@@ -5608,7 +5847,7 @@
       <c r="R99" s="3"/>
       <c r="S99" s="3"/>
     </row>
-    <row r="100" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="14"/>
       <c r="B100" s="31"/>
       <c r="C100" s="28"/>
@@ -5629,7 +5868,7 @@
       <c r="R100" s="3"/>
       <c r="S100" s="3"/>
     </row>
-    <row r="101" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="14"/>
       <c r="B101" s="31"/>
       <c r="C101" s="28"/>
@@ -5650,7 +5889,7 @@
       <c r="R101" s="3"/>
       <c r="S101" s="3"/>
     </row>
-    <row r="102" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="14"/>
       <c r="B102" s="31"/>
       <c r="C102" s="28"/>
@@ -5671,7 +5910,7 @@
       <c r="R102" s="3"/>
       <c r="S102" s="3"/>
     </row>
-    <row r="103" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="14"/>
       <c r="B103" s="31"/>
       <c r="C103" s="28"/>
@@ -5692,7 +5931,7 @@
       <c r="R103" s="3"/>
       <c r="S103" s="3"/>
     </row>
-    <row r="104" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="14"/>
       <c r="B104" s="31"/>
       <c r="C104" s="28"/>
@@ -5713,7 +5952,7 @@
       <c r="R104" s="3"/>
       <c r="S104" s="3"/>
     </row>
-    <row r="105" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="14"/>
       <c r="B105" s="31"/>
       <c r="C105" s="28"/>
@@ -5734,7 +5973,7 @@
       <c r="R105" s="3"/>
       <c r="S105" s="3"/>
     </row>
-    <row r="106" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="14"/>
       <c r="B106" s="31"/>
       <c r="C106" s="28"/>
@@ -5755,7 +5994,7 @@
       <c r="R106" s="3"/>
       <c r="S106" s="3"/>
     </row>
-    <row r="107" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A107" s="14"/>
       <c r="B107" s="31"/>
       <c r="C107" s="28"/>
@@ -5776,7 +6015,7 @@
       <c r="R107" s="3"/>
       <c r="S107" s="3"/>
     </row>
-    <row r="108" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A108" s="14"/>
       <c r="B108" s="31"/>
       <c r="C108" s="28"/>
@@ -5797,7 +6036,7 @@
       <c r="R108" s="3"/>
       <c r="S108" s="3"/>
     </row>
-    <row r="109" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A109" s="14"/>
       <c r="B109" s="31"/>
       <c r="C109" s="28"/>
@@ -5818,7 +6057,7 @@
       <c r="R109" s="3"/>
       <c r="S109" s="3"/>
     </row>
-    <row r="110" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="14"/>
       <c r="B110" s="31"/>
       <c r="C110" s="28"/>
@@ -5839,7 +6078,7 @@
       <c r="R110" s="3"/>
       <c r="S110" s="3"/>
     </row>
-    <row r="111" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="14"/>
       <c r="B111" s="31"/>
       <c r="C111" s="28"/>
@@ -5860,7 +6099,7 @@
       <c r="R111" s="3"/>
       <c r="S111" s="3"/>
     </row>
-    <row r="112" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A112" s="14"/>
       <c r="B112" s="31"/>
       <c r="C112" s="28"/>
@@ -5881,7 +6120,7 @@
       <c r="R112" s="3"/>
       <c r="S112" s="3"/>
     </row>
-    <row r="113" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A113" s="14"/>
       <c r="B113" s="31"/>
       <c r="C113" s="28"/>
@@ -5902,7 +6141,7 @@
       <c r="R113" s="3"/>
       <c r="S113" s="3"/>
     </row>
-    <row r="114" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="14"/>
       <c r="B114" s="31"/>
       <c r="C114" s="28"/>
@@ -5923,7 +6162,7 @@
       <c r="R114" s="3"/>
       <c r="S114" s="3"/>
     </row>
-    <row r="115" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A115" s="14"/>
       <c r="B115" s="31"/>
       <c r="C115" s="28"/>
@@ -5944,7 +6183,7 @@
       <c r="R115" s="3"/>
       <c r="S115" s="3"/>
     </row>
-    <row r="116" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A116" s="14"/>
       <c r="B116" s="31"/>
       <c r="C116" s="28"/>
@@ -5965,7 +6204,7 @@
       <c r="R116" s="3"/>
       <c r="S116" s="3"/>
     </row>
-    <row r="117" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A117" s="14"/>
       <c r="B117" s="31"/>
       <c r="C117" s="28"/>
@@ -5986,7 +6225,7 @@
       <c r="R117" s="3"/>
       <c r="S117" s="3"/>
     </row>
-    <row r="118" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A118" s="14"/>
       <c r="B118" s="31"/>
       <c r="C118" s="28"/>
@@ -6007,7 +6246,7 @@
       <c r="R118" s="3"/>
       <c r="S118" s="3"/>
     </row>
-    <row r="119" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A119" s="14"/>
       <c r="B119" s="31"/>
       <c r="C119" s="28"/>
@@ -6028,7 +6267,7 @@
       <c r="R119" s="3"/>
       <c r="S119" s="3"/>
     </row>
-    <row r="120" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A120" s="14"/>
       <c r="B120" s="31"/>
       <c r="C120" s="28"/>
@@ -6049,7 +6288,7 @@
       <c r="R120" s="3"/>
       <c r="S120" s="3"/>
     </row>
-    <row r="121" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A121" s="14"/>
       <c r="B121" s="31"/>
       <c r="C121" s="28"/>
@@ -6070,7 +6309,7 @@
       <c r="R121" s="3"/>
       <c r="S121" s="3"/>
     </row>
-    <row r="122" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A122" s="14"/>
       <c r="B122" s="31"/>
       <c r="C122" s="28"/>
@@ -6091,7 +6330,7 @@
       <c r="R122" s="3"/>
       <c r="S122" s="3"/>
     </row>
-    <row r="123" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A123" s="14"/>
       <c r="B123" s="31"/>
       <c r="C123" s="28"/>
@@ -6112,7 +6351,7 @@
       <c r="R123" s="3"/>
       <c r="S123" s="3"/>
     </row>
-    <row r="124" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A124" s="14"/>
       <c r="B124" s="31"/>
       <c r="C124" s="28"/>
@@ -6133,7 +6372,7 @@
       <c r="R124" s="3"/>
       <c r="S124" s="3"/>
     </row>
-    <row r="125" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A125" s="14"/>
       <c r="B125" s="31"/>
       <c r="C125" s="28"/>
@@ -6154,7 +6393,7 @@
       <c r="R125" s="3"/>
       <c r="S125" s="3"/>
     </row>
-    <row r="126" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" s="14"/>
       <c r="B126" s="31"/>
       <c r="C126" s="28"/>
@@ -6175,7 +6414,7 @@
       <c r="R126" s="3"/>
       <c r="S126" s="3"/>
     </row>
-    <row r="127" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A127" s="14"/>
       <c r="B127" s="31"/>
       <c r="C127" s="28"/>
@@ -6196,7 +6435,7 @@
       <c r="R127" s="3"/>
       <c r="S127" s="3"/>
     </row>
-    <row r="128" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A128" s="14"/>
       <c r="B128" s="31"/>
       <c r="C128" s="28"/>
@@ -6217,7 +6456,7 @@
       <c r="R128" s="3"/>
       <c r="S128" s="3"/>
     </row>
-    <row r="129" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A129" s="14"/>
       <c r="B129" s="31"/>
       <c r="C129" s="28"/>
@@ -6238,7 +6477,7 @@
       <c r="R129" s="3"/>
       <c r="S129" s="3"/>
     </row>
-    <row r="130" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" s="14"/>
       <c r="B130" s="31"/>
       <c r="C130" s="28"/>
@@ -6259,7 +6498,7 @@
       <c r="R130" s="3"/>
       <c r="S130" s="3"/>
     </row>
-    <row r="131" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A131" s="14"/>
       <c r="B131" s="31"/>
       <c r="C131" s="28"/>
@@ -6280,7 +6519,7 @@
       <c r="R131" s="3"/>
       <c r="S131" s="3"/>
     </row>
-    <row r="132" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:19" ht="14.85" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A132" s="14"/>
       <c r="B132" s="31"/>
       <c r="C132" s="28"/>
@@ -6302,6 +6541,9 @@
       <c r="S132" s="3"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="E90:E91"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
   <headerFooter>

</xml_diff>

<commit_message>
updated fuselage wetted area
</commit_message>
<xml_diff>
--- a/SizingParams.xlsx
+++ b/SizingParams.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\Desktop\Fall 2026\AAE 451\451-DBF-Team01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6264661C-07D5-4B6E-9648-D59E06C92932}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60007970-5A4F-400B-B565-6CA8D1228FE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1467,7 +1467,7 @@
         <v>56</v>
       </c>
       <c r="C28">
-        <v>0.24299999999999999</v>
+        <v>0.433</v>
       </c>
       <c r="D28" t="s">
         <v>66</v>

</xml_diff>

<commit_message>
V-n, Wing, Tail, Fuselage, Takoff rotation First pass
ff
</commit_message>
<xml_diff>
--- a/SizingParams.xlsx
+++ b/SizingParams.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ceaa8977d2236823/Documents/GitHub/451-DBF-Team01/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="273" documentId="13_ncr:1_{60007970-5A4F-400B-B565-6CA8D1228FE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2540A57B-32A3-4A49-866F-5AA261EF41B3}"/>
+  <xr:revisionPtr revIDLastSave="340" documentId="13_ncr:1_{60007970-5A4F-400B-B565-6CA8D1228FE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17327AF0-D2A2-401A-AFA4-5BA44D815C39}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="306">
   <si>
     <t>Parameter</t>
   </si>
@@ -892,9 +892,6 @@
     <t>Mass_g</t>
   </si>
   <si>
-    <t>Station_m</t>
-  </si>
-  <si>
     <t>Propeller+spinner</t>
   </si>
   <si>
@@ -946,13 +943,16 @@
     <t>Servo, rudder</t>
   </si>
   <si>
-    <t>H-tail (spar+foam)</t>
-  </si>
-  <si>
     <t>V-tail (spar+foam)</t>
   </si>
   <si>
-    <t>PLACEHOLDER, rescaled to match iterated MTOM</t>
+    <t>Height_m</t>
+  </si>
+  <si>
+    <t>Horizontal tail (spar+foam)</t>
+  </si>
+  <si>
+    <t>X_m</t>
   </si>
 </sst>
 </file>
@@ -1407,8 +1407,8 @@
     <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="10.6640625" customWidth="1"/>
-    <col min="5" max="5" width="44" customWidth="1"/>
-    <col min="6" max="6" width="60" customWidth="1"/>
+    <col min="5" max="5" width="168.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
@@ -3194,6 +3194,7 @@
   <cols>
     <col min="1" max="1" width="32.5546875" customWidth="1"/>
     <col min="2" max="3" width="32.5546875" style="21" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" style="21" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -3204,15 +3205,15 @@
         <v>284</v>
       </c>
       <c r="C1" s="20" t="s">
-        <v>285</v>
-      </c>
-      <c r="D1" t="s">
-        <v>5</v>
+        <v>305</v>
+      </c>
+      <c r="D1" s="21" t="s">
+        <v>303</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B2" s="22">
         <v>25.9</v>
@@ -3220,13 +3221,13 @@
       <c r="C2" s="22">
         <v>0</v>
       </c>
-      <c r="D2" t="s">
-        <v>305</v>
+      <c r="D2" s="22">
+        <v>2.8000000000000001E-2</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B3" s="22">
         <v>116.7</v>
@@ -3234,13 +3235,13 @@
       <c r="C3" s="22">
         <v>3.5000000000000003E-2</v>
       </c>
-      <c r="D3" t="s">
-        <v>305</v>
+      <c r="D3" s="22">
+        <v>2.8000000000000001E-2</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B4" s="22">
         <v>22.7</v>
@@ -3248,13 +3249,13 @@
       <c r="C4" s="22">
         <v>5.5E-2</v>
       </c>
-      <c r="D4" t="s">
-        <v>305</v>
+      <c r="D4" s="22">
+        <v>2.8000000000000001E-2</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B5" s="22">
         <v>32.4</v>
@@ -3262,13 +3263,13 @@
       <c r="C5" s="22">
         <v>0.09</v>
       </c>
-      <c r="D5" t="s">
-        <v>305</v>
+      <c r="D5" s="22">
+        <v>2.5000000000000001E-2</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B6" s="22">
         <v>45.4</v>
@@ -3276,13 +3277,13 @@
       <c r="C6" s="22">
         <v>9.5000000000000001E-2</v>
       </c>
-      <c r="D6" t="s">
-        <v>305</v>
+      <c r="D6" s="22">
+        <v>-4.4999999999999998E-2</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B7" s="22">
         <v>440.8</v>
@@ -3290,13 +3291,13 @@
       <c r="C7" s="22">
         <v>0.12</v>
       </c>
-      <c r="D7" t="s">
-        <v>305</v>
+      <c r="D7" s="22">
+        <v>1.4999999999999999E-2</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B8" s="22">
         <v>58.3</v>
@@ -3304,13 +3305,13 @@
       <c r="C8" s="22">
         <v>0.23</v>
       </c>
-      <c r="D8" t="s">
-        <v>305</v>
+      <c r="D8" s="22">
+        <v>2.8000000000000001E-2</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B9" s="22">
         <v>64.8</v>
@@ -3318,13 +3319,13 @@
       <c r="C9" s="22">
         <v>0.3</v>
       </c>
-      <c r="D9" t="s">
-        <v>305</v>
+      <c r="D9" s="22">
+        <v>2.8000000000000001E-2</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B10" s="22">
         <v>259.3</v>
@@ -3332,13 +3333,13 @@
       <c r="C10" s="22">
         <v>0.32</v>
       </c>
-      <c r="D10" t="s">
-        <v>305</v>
+      <c r="D10" s="22">
+        <v>2.8000000000000001E-2</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B11" s="22">
         <v>13.4</v>
@@ -3346,10 +3347,13 @@
       <c r="C11" s="22">
         <v>0.4</v>
       </c>
+      <c r="D11" s="22">
+        <v>5.5E-2</v>
+      </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B12" s="22">
         <v>13.4</v>
@@ -3357,10 +3361,13 @@
       <c r="C12" s="22">
         <v>0.4</v>
       </c>
+      <c r="D12" s="22">
+        <v>5.5E-2</v>
+      </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B13" s="21">
         <v>520</v>
@@ -3368,10 +3375,13 @@
       <c r="C13" s="22">
         <v>0.4</v>
       </c>
+      <c r="D13" s="22">
+        <v>2.8000000000000001E-2</v>
+      </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B14" s="22">
         <v>907.6</v>
@@ -3379,13 +3389,13 @@
       <c r="C14" s="22">
         <v>0.40699999999999997</v>
       </c>
-      <c r="D14" t="s">
-        <v>305</v>
+      <c r="D14" s="22">
+        <v>5.5E-2</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B15" s="22">
         <v>142.6</v>
@@ -3393,13 +3403,13 @@
       <c r="C15" s="22">
         <v>0.43</v>
       </c>
-      <c r="D15" t="s">
-        <v>305</v>
+      <c r="D15" s="22">
+        <v>-7.8E-2</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B16" s="22">
         <v>1231.8</v>
@@ -3407,13 +3417,13 @@
       <c r="C16" s="22">
         <v>0.55000000000000004</v>
       </c>
-      <c r="D16" t="s">
-        <v>305</v>
+      <c r="D16" s="22">
+        <v>2.8000000000000001E-2</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B17" s="22">
         <v>13.4</v>
@@ -3421,10 +3431,13 @@
       <c r="C17" s="22">
         <v>1</v>
       </c>
+      <c r="D17" s="22">
+        <v>1.4999999999999999E-2</v>
+      </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B18" s="22">
         <v>13.4</v>
@@ -3432,10 +3445,13 @@
       <c r="C18" s="22">
         <v>1</v>
       </c>
+      <c r="D18" s="22">
+        <v>1.4999999999999999E-2</v>
+      </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B19" s="22">
         <v>77.8</v>
@@ -3443,13 +3459,13 @@
       <c r="C19" s="22">
         <v>1.05</v>
       </c>
-      <c r="D19" t="s">
-        <v>305</v>
+      <c r="D19" s="22">
+        <v>1.4999999999999999E-2</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="B20" s="22">
         <v>51.9</v>
@@ -3457,8 +3473,8 @@
       <c r="C20" s="22">
         <v>1.05</v>
       </c>
-      <c r="D20" t="s">
-        <v>305</v>
+      <c r="D20" s="22">
+        <v>0.15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
pushy pushy; mir makes me horny
</commit_message>
<xml_diff>
--- a/SizingParams.xlsx
+++ b/SizingParams.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ceaa8977d2236823/Documents/GitHub/451-DBF-Team01/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hudson/Documents/GitHub/451-DBF-Team01/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="340" documentId="13_ncr:1_{60007970-5A4F-400B-B565-6CA8D1228FE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17327AF0-D2A2-401A-AFA4-5BA44D815C39}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B07C9115-910C-EA49-AF5C-D506317D2282}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -976,6 +976,7 @@
       <sz val="11"/>
       <color indexed="8"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -1401,17 +1402,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F104"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="10.6640625" customWidth="1"/>
-    <col min="5" max="5" width="168.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="168.1640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1431,7 +1432,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1448,7 +1449,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -1465,7 +1466,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1482,7 +1483,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -1499,7 +1500,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -1516,7 +1517,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -1533,7 +1534,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>20</v>
       </c>
@@ -1550,7 +1551,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>205</v>
       </c>
@@ -1564,7 +1565,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1581,7 +1582,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -1598,7 +1599,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>27</v>
       </c>
@@ -1615,7 +1616,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>28</v>
       </c>
@@ -1632,7 +1633,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>31</v>
       </c>
@@ -1649,7 +1650,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>33</v>
       </c>
@@ -1666,7 +1667,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>35</v>
       </c>
@@ -1683,7 +1684,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>37</v>
       </c>
@@ -1700,7 +1701,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>39</v>
       </c>
@@ -1717,7 +1718,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>41</v>
       </c>
@@ -1734,7 +1735,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>45</v>
       </c>
@@ -1751,7 +1752,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>48</v>
       </c>
@@ -1768,7 +1769,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>51</v>
       </c>
@@ -1785,7 +1786,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>53</v>
       </c>
@@ -1802,7 +1803,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>55</v>
       </c>
@@ -1819,7 +1820,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>58</v>
       </c>
@@ -1836,7 +1837,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>61</v>
       </c>
@@ -1853,7 +1854,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>63</v>
       </c>
@@ -1870,7 +1871,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>65</v>
       </c>
@@ -1887,7 +1888,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>68</v>
       </c>
@@ -1904,7 +1905,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>70</v>
       </c>
@@ -1921,7 +1922,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>72</v>
       </c>
@@ -1938,7 +1939,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>74</v>
       </c>
@@ -1955,7 +1956,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>76</v>
       </c>
@@ -1972,7 +1973,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>78</v>
       </c>
@@ -1989,7 +1990,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>80</v>
       </c>
@@ -2006,7 +2007,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>82</v>
       </c>
@@ -2023,7 +2024,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>84</v>
       </c>
@@ -2040,7 +2041,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>86</v>
       </c>
@@ -2057,7 +2058,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>88</v>
       </c>
@@ -2074,7 +2075,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>90</v>
       </c>
@@ -2091,7 +2092,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>92</v>
       </c>
@@ -2108,7 +2109,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>94</v>
       </c>
@@ -2125,7 +2126,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>96</v>
       </c>
@@ -2142,7 +2143,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>98</v>
       </c>
@@ -2159,7 +2160,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>100</v>
       </c>
@@ -2176,7 +2177,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>103</v>
       </c>
@@ -2193,7 +2194,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>105</v>
       </c>
@@ -2210,7 +2211,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>107</v>
       </c>
@@ -2227,7 +2228,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>109</v>
       </c>
@@ -2244,7 +2245,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>111</v>
       </c>
@@ -2252,7 +2253,7 @@
         <v>56</v>
       </c>
       <c r="C50">
-        <v>0.23</v>
+        <v>0.17</v>
       </c>
       <c r="D50" t="s">
         <v>8</v>
@@ -2261,7 +2262,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>113</v>
       </c>
@@ -2278,7 +2279,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>115</v>
       </c>
@@ -2295,7 +2296,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>117</v>
       </c>
@@ -2312,7 +2313,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>119</v>
       </c>
@@ -2329,7 +2330,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>121</v>
       </c>
@@ -2346,7 +2347,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>123</v>
       </c>
@@ -2363,7 +2364,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>125</v>
       </c>
@@ -2380,7 +2381,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>127</v>
       </c>
@@ -2397,7 +2398,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>129</v>
       </c>
@@ -2414,7 +2415,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>131</v>
       </c>
@@ -2431,7 +2432,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>133</v>
       </c>
@@ -2448,7 +2449,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>135</v>
       </c>
@@ -2465,7 +2466,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>139</v>
       </c>
@@ -2482,7 +2483,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>141</v>
       </c>
@@ -2499,7 +2500,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>143</v>
       </c>
@@ -2516,7 +2517,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>145</v>
       </c>
@@ -2533,7 +2534,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>201</v>
       </c>
@@ -2550,7 +2551,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>146</v>
       </c>
@@ -2567,7 +2568,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>148</v>
       </c>
@@ -2584,7 +2585,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>150</v>
       </c>
@@ -2601,7 +2602,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>152</v>
       </c>
@@ -2618,7 +2619,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>154</v>
       </c>
@@ -2635,7 +2636,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>157</v>
       </c>
@@ -2652,7 +2653,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>160</v>
       </c>
@@ -2669,7 +2670,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>162</v>
       </c>
@@ -2686,7 +2687,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>165</v>
       </c>
@@ -2703,7 +2704,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>167</v>
       </c>
@@ -2720,7 +2721,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>169</v>
       </c>
@@ -2737,7 +2738,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>172</v>
       </c>
@@ -2754,7 +2755,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>174</v>
       </c>
@@ -2771,7 +2772,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>176</v>
       </c>
@@ -2788,7 +2789,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>178</v>
       </c>
@@ -2805,7 +2806,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>180</v>
       </c>
@@ -2822,7 +2823,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>183</v>
       </c>
@@ -2839,7 +2840,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>186</v>
       </c>
@@ -2856,7 +2857,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>189</v>
       </c>
@@ -2873,7 +2874,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>191</v>
       </c>
@@ -2890,7 +2891,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>193</v>
       </c>
@@ -2907,7 +2908,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>196</v>
       </c>
@@ -2924,7 +2925,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>198</v>
       </c>
@@ -2941,7 +2942,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>248</v>
       </c>
@@ -2958,7 +2959,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>251</v>
       </c>
@@ -2975,7 +2976,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>253</v>
       </c>
@@ -2992,7 +2993,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>255</v>
       </c>
@@ -3009,7 +3010,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>261</v>
       </c>
@@ -3026,7 +3027,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>263</v>
       </c>
@@ -3043,7 +3044,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>265</v>
       </c>
@@ -3060,7 +3061,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>268</v>
       </c>
@@ -3077,7 +3078,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>270</v>
       </c>
@@ -3094,7 +3095,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>272</v>
       </c>
@@ -3111,7 +3112,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>274</v>
       </c>
@@ -3128,7 +3129,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>276</v>
       </c>
@@ -3145,7 +3146,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>278</v>
       </c>
@@ -3162,7 +3163,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>280</v>
       </c>
@@ -3190,14 +3191,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFCC8514-E0AF-4C67-BF86-8649FC702924}">
   <dimension ref="A1:D20"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="32.5546875" customWidth="1"/>
-    <col min="2" max="3" width="32.5546875" style="21" customWidth="1"/>
+    <col min="1" max="1" width="32.5" customWidth="1"/>
+    <col min="2" max="3" width="32.5" style="21" customWidth="1"/>
     <col min="4" max="4" width="13.33203125" style="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="18" t="s">
         <v>283</v>
       </c>
@@ -3211,7 +3212,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>285</v>
       </c>
@@ -3225,7 +3226,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>286</v>
       </c>
@@ -3239,7 +3240,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>287</v>
       </c>
@@ -3253,7 +3254,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>288</v>
       </c>
@@ -3267,7 +3268,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>289</v>
       </c>
@@ -3281,7 +3282,7 @@
         <v>-4.4999999999999998E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>290</v>
       </c>
@@ -3295,7 +3296,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>291</v>
       </c>
@@ -3309,7 +3310,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>292</v>
       </c>
@@ -3323,7 +3324,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>293</v>
       </c>
@@ -3337,7 +3338,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>294</v>
       </c>
@@ -3351,7 +3352,7 @@
         <v>5.5E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>295</v>
       </c>
@@ -3365,7 +3366,7 @@
         <v>5.5E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>296</v>
       </c>
@@ -3379,7 +3380,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>297</v>
       </c>
@@ -3393,7 +3394,7 @@
         <v>5.5E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>298</v>
       </c>
@@ -3407,7 +3408,7 @@
         <v>-7.8E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>299</v>
       </c>
@@ -3421,7 +3422,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>300</v>
       </c>
@@ -3435,7 +3436,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>301</v>
       </c>
@@ -3449,7 +3450,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>304</v>
       </c>
@@ -3463,7 +3464,7 @@
         <v>1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>302</v>
       </c>
@@ -3485,26 +3486,26 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{118BE621-EF6B-4648-868E-9937B9C5B685}">
   <dimension ref="A1:F32"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="48.109375" style="2" customWidth="1"/>
-    <col min="2" max="4" width="15.77734375" style="2" customWidth="1"/>
-    <col min="5" max="5" width="3.77734375" style="2" customWidth="1"/>
-    <col min="6" max="6" width="46.77734375" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="8.88671875" style="2"/>
+    <col min="1" max="1" width="48.1640625" style="2" customWidth="1"/>
+    <col min="2" max="4" width="15.83203125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="3.83203125" style="2" customWidth="1"/>
+    <col min="6" max="6" width="46.83203125" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>208</v>
       </c>
@@ -3518,7 +3519,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>212</v>
       </c>
@@ -3536,7 +3537,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>214</v>
       </c>
@@ -3556,7 +3557,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>216</v>
       </c>
@@ -3576,7 +3577,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>217</v>
       </c>
@@ -3594,7 +3595,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>218</v>
       </c>
@@ -3614,7 +3615,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>220</v>
       </c>
@@ -3631,7 +3632,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>222</v>
       </c>
@@ -3648,7 +3649,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>223</v>
       </c>
@@ -3668,7 +3669,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>225</v>
       </c>
@@ -3685,7 +3686,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>257</v>
       </c>
@@ -3705,7 +3706,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>258</v>
       </c>
@@ -3725,7 +3726,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
         <v>227</v>
       </c>
@@ -3733,7 +3734,7 @@
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>228</v>
       </c>
@@ -3750,7 +3751,7 @@
         <v>1.9823131728623846</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>229</v>
       </c>
@@ -3767,7 +3768,7 @@
         <v>1.1592794807274085</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>230</v>
       </c>
@@ -3784,7 +3785,7 @@
         <v>-0.62740704594148844</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>231</v>
       </c>
@@ -3801,7 +3802,7 @@
         <v>-0.96540266006846076</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
         <v>232</v>
       </c>
@@ -3809,7 +3810,7 @@
       <c r="C21" s="4"/>
       <c r="D21" s="4"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>233</v>
       </c>
@@ -3826,7 +3827,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>234</v>
       </c>
@@ -3843,7 +3844,7 @@
         <v>0.52359877559829882</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>235</v>
       </c>
@@ -3860,7 +3861,7 @@
         <v>-0.50548365077118673</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>236</v>
       </c>
@@ -3877,7 +3878,7 @@
         <v>324.01250000000005</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>237</v>
       </c>
@@ -3894,7 +3895,7 @@
         <v>1.42884E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" s="11" t="s">
         <v>238</v>
       </c>
@@ -3911,7 +3912,7 @@
         <v>-0.13760360258695806</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>239</v>
       </c>
@@ -3928,7 +3929,7 @@
         <v>0.13760360258695806</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" s="11" t="s">
         <v>240</v>
       </c>
@@ -3945,7 +3946,7 @@
         <v>22.925083964169769</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>241</v>
       </c>
@@ -3953,7 +3954,7 @@
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>242</v>
       </c>
@@ -3961,7 +3962,7 @@
       <c r="C31" s="14"/>
       <c r="D31" s="14"/>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>243</v>
       </c>

</xml_diff>

<commit_message>
I have a rubber band around my balls
</commit_message>
<xml_diff>
--- a/SizingParams.xlsx
+++ b/SizingParams.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ceaa8977d2236823/Documents/GitHub/451-DBF-Team01/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\Desktop\Fall 2026\AAE 451\451-DBF-Team01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{5D9A45EA-EF47-47B7-862F-774A8D1C5EE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FFB324C3-D317-425C-8AED-9FBC36E04367}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{574AC2E1-1736-470D-86C8-2E394B026491}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1173" uniqueCount="563">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1176" uniqueCount="564">
   <si>
     <t>Parameter</t>
   </si>
@@ -1726,6 +1726,9 @@
   </si>
   <si>
     <t>bolt_OD</t>
+  </si>
+  <si>
+    <t>T_static_actual</t>
   </si>
 </sst>
 </file>
@@ -1878,7 +1881,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
@@ -1925,9 +1928,6 @@
     <xf numFmtId="1" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1960,10 +1960,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:F146" totalsRowShown="0">
-  <autoFilter ref="A1:F146" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:F147" totalsRowShown="0">
+  <autoFilter ref="A1:F147" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E43">
-    <sortCondition ref="B1:B101"/>
+    <sortCondition ref="B1:B102"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Parameter"/>
@@ -2240,18 +2240,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F132"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F133"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.109375" style="20" customWidth="1"/>
-    <col min="3" max="3" width="13.6640625" style="20" customWidth="1"/>
-    <col min="4" max="4" width="16.88671875" style="20" customWidth="1"/>
-    <col min="5" max="5" width="168.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="142.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" style="20" customWidth="1"/>
+    <col min="3" max="3" width="13.7109375" style="20" customWidth="1"/>
+    <col min="4" max="4" width="16.85546875" style="20" customWidth="1"/>
+    <col min="5" max="5" width="168.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="142.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2271,7 +2271,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -2288,7 +2288,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -2305,7 +2305,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -2322,7 +2322,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -2339,7 +2339,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -2356,7 +2356,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -2373,7 +2373,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>20</v>
       </c>
@@ -2390,7 +2390,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>203</v>
       </c>
@@ -2404,7 +2404,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -2421,7 +2421,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -2438,7 +2438,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>27</v>
       </c>
@@ -2455,7 +2455,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>28</v>
       </c>
@@ -2472,7 +2472,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>31</v>
       </c>
@@ -2489,7 +2489,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>33</v>
       </c>
@@ -2506,7 +2506,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>35</v>
       </c>
@@ -2523,7 +2523,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>37</v>
       </c>
@@ -2540,7 +2540,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>39</v>
       </c>
@@ -2557,7 +2557,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>41</v>
       </c>
@@ -2574,7 +2574,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>45</v>
       </c>
@@ -2591,7 +2591,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>48</v>
       </c>
@@ -2608,7 +2608,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>51</v>
       </c>
@@ -2625,7 +2625,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>53</v>
       </c>
@@ -2642,7 +2642,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>55</v>
       </c>
@@ -2659,7 +2659,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>58</v>
       </c>
@@ -2676,7 +2676,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>61</v>
       </c>
@@ -2693,7 +2693,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>63</v>
       </c>
@@ -2710,7 +2710,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>65</v>
       </c>
@@ -2727,7 +2727,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>68</v>
       </c>
@@ -2744,7 +2744,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>70</v>
       </c>
@@ -2761,7 +2761,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>72</v>
       </c>
@@ -2778,7 +2778,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>74</v>
       </c>
@@ -2795,7 +2795,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>76</v>
       </c>
@@ -2812,7 +2812,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>78</v>
       </c>
@@ -2829,7 +2829,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>80</v>
       </c>
@@ -2846,7 +2846,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>82</v>
       </c>
@@ -2863,7 +2863,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>84</v>
       </c>
@@ -2880,7 +2880,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>86</v>
       </c>
@@ -2897,7 +2897,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>88</v>
       </c>
@@ -2914,7 +2914,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>89</v>
       </c>
@@ -2931,7 +2931,7 @@
         <v>521</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>90</v>
       </c>
@@ -2948,7 +2948,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>92</v>
       </c>
@@ -2965,7 +2965,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>94</v>
       </c>
@@ -2982,7 +2982,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>96</v>
       </c>
@@ -2999,7 +2999,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>98</v>
       </c>
@@ -3016,7 +3016,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>101</v>
       </c>
@@ -3033,7 +3033,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>103</v>
       </c>
@@ -3050,7 +3050,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>105</v>
       </c>
@@ -3067,7 +3067,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>107</v>
       </c>
@@ -3084,7 +3084,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>109</v>
       </c>
@@ -3101,7 +3101,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>111</v>
       </c>
@@ -3118,7 +3118,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>113</v>
       </c>
@@ -3135,7 +3135,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>115</v>
       </c>
@@ -3152,7 +3152,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>117</v>
       </c>
@@ -3169,7 +3169,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>119</v>
       </c>
@@ -3186,7 +3186,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>121</v>
       </c>
@@ -3203,7 +3203,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>123</v>
       </c>
@@ -3220,7 +3220,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>125</v>
       </c>
@@ -3237,7 +3237,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>127</v>
       </c>
@@ -3254,7 +3254,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>129</v>
       </c>
@@ -3271,7 +3271,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>131</v>
       </c>
@@ -3288,7 +3288,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>133</v>
       </c>
@@ -3305,7 +3305,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>137</v>
       </c>
@@ -3322,7 +3322,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>139</v>
       </c>
@@ -3339,7 +3339,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>141</v>
       </c>
@@ -3356,7 +3356,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>143</v>
       </c>
@@ -3373,7 +3373,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>199</v>
       </c>
@@ -3390,7 +3390,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>144</v>
       </c>
@@ -3407,7 +3407,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>146</v>
       </c>
@@ -3424,7 +3424,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>148</v>
       </c>
@@ -3441,7 +3441,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>150</v>
       </c>
@@ -3458,7 +3458,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>152</v>
       </c>
@@ -3475,7 +3475,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>155</v>
       </c>
@@ -3492,7 +3492,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>158</v>
       </c>
@@ -3509,7 +3509,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>160</v>
       </c>
@@ -3526,7 +3526,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>163</v>
       </c>
@@ -3543,7 +3543,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>165</v>
       </c>
@@ -3560,7 +3560,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>167</v>
       </c>
@@ -3577,7 +3577,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>170</v>
       </c>
@@ -3594,7 +3594,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>172</v>
       </c>
@@ -3611,7 +3611,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>174</v>
       </c>
@@ -3628,7 +3628,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>176</v>
       </c>
@@ -3645,7 +3645,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>178</v>
       </c>
@@ -3662,7 +3662,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>181</v>
       </c>
@@ -3679,7 +3679,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>184</v>
       </c>
@@ -3696,7 +3696,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>187</v>
       </c>
@@ -3713,7 +3713,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>189</v>
       </c>
@@ -3730,7 +3730,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>191</v>
       </c>
@@ -3747,7 +3747,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>194</v>
       </c>
@@ -3764,7 +3764,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>196</v>
       </c>
@@ -3781,162 +3781,160 @@
         <v>197</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
+        <v>563</v>
+      </c>
+      <c r="B91" s="20" t="s">
+        <v>168</v>
+      </c>
+      <c r="C91" s="20">
+        <f>2.085*9.81</f>
+        <v>20.453849999999999</v>
+      </c>
+      <c r="D91" s="20" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
         <v>246</v>
-      </c>
-      <c r="B91" s="20" t="s">
-        <v>247</v>
-      </c>
-      <c r="C91" s="20">
-        <v>1</v>
-      </c>
-      <c r="D91" s="20" t="s">
-        <v>8</v>
-      </c>
-      <c r="E91" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A92" t="s">
-        <v>249</v>
       </c>
       <c r="B92" s="20" t="s">
         <v>247</v>
       </c>
       <c r="C92" s="20">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="D92" s="20" t="s">
         <v>8</v>
       </c>
       <c r="E92" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B93" s="20" t="s">
         <v>247</v>
       </c>
       <c r="C93" s="20">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="D93" s="20" t="s">
         <v>8</v>
       </c>
       <c r="E93" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="B94" s="20" t="s">
         <v>247</v>
       </c>
       <c r="C94" s="20">
-        <v>0.85</v>
+        <v>1</v>
       </c>
       <c r="D94" s="20" t="s">
         <v>8</v>
       </c>
       <c r="E94" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="B95" s="20" t="s">
         <v>247</v>
       </c>
       <c r="C95" s="20">
+        <v>0.85</v>
+      </c>
+      <c r="D95" s="20" t="s">
+        <v>8</v>
+      </c>
+      <c r="E95" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>259</v>
+      </c>
+      <c r="B96" s="20" t="s">
+        <v>247</v>
+      </c>
+      <c r="C96" s="20">
         <v>5.5</v>
       </c>
-      <c r="D95" s="20" t="s">
+      <c r="D96" s="20" t="s">
         <v>188</v>
       </c>
-      <c r="E95" t="s">
+      <c r="E96" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A96" t="s">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
         <v>261</v>
       </c>
-      <c r="B96" s="20" t="s">
+      <c r="B97" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="C96" s="20">
+      <c r="C97" s="20">
         <v>-0.66</v>
-      </c>
-      <c r="D96" s="20" t="s">
-        <v>8</v>
-      </c>
-      <c r="E96" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A97" t="s">
-        <v>262</v>
-      </c>
-      <c r="B97" s="27" t="s">
-        <v>263</v>
-      </c>
-      <c r="C97" s="27">
-        <v>0.25</v>
       </c>
       <c r="D97" s="20" t="s">
         <v>8</v>
       </c>
       <c r="E97" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>264</v>
-      </c>
-      <c r="B98" s="30" t="s">
+        <v>262</v>
+      </c>
+      <c r="B98" s="27" t="s">
         <v>263</v>
       </c>
-      <c r="C98" s="30">
-        <v>1</v>
+      <c r="C98" s="27">
+        <v>0.25</v>
       </c>
       <c r="D98" s="20" t="s">
         <v>8</v>
       </c>
       <c r="E98" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>265</v>
-      </c>
-      <c r="B99" s="30" t="s">
+        <v>264</v>
+      </c>
+      <c r="B99" s="20" t="s">
         <v>263</v>
       </c>
-      <c r="C99" s="30">
+      <c r="C99" s="20">
         <v>1</v>
       </c>
       <c r="D99" s="20" t="s">
         <v>8</v>
       </c>
       <c r="E99" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B100" s="20" t="s">
         <v>263</v>
@@ -3948,524 +3946,541 @@
         <v>8</v>
       </c>
       <c r="E100" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>266</v>
+      </c>
+      <c r="B101" s="20" t="s">
+        <v>263</v>
+      </c>
+      <c r="C101" s="20">
+        <v>1</v>
+      </c>
+      <c r="D101" s="20" t="s">
+        <v>8</v>
+      </c>
+      <c r="E101" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A101" t="s">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
         <v>267</v>
       </c>
-      <c r="B101" s="27" t="s">
+      <c r="B102" s="27" t="s">
         <v>263</v>
       </c>
-      <c r="C101" s="27">
+      <c r="C102" s="27">
         <v>1.2699999999999999E-2</v>
-      </c>
-      <c r="D101" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="E101" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A102" t="s">
-        <v>268</v>
-      </c>
-      <c r="B102" s="28" t="s">
-        <v>263</v>
-      </c>
-      <c r="C102" s="28">
-        <v>0.29499999999999998</v>
       </c>
       <c r="D102" s="20" t="s">
         <v>59</v>
       </c>
       <c r="E102" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>268</v>
+      </c>
+      <c r="B103" s="28" t="s">
+        <v>263</v>
+      </c>
+      <c r="C103" s="28">
+        <v>0.29499999999999998</v>
+      </c>
+      <c r="D103" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="E103" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A103" t="s">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
         <v>269</v>
       </c>
-      <c r="B103" s="20" t="s">
+      <c r="B104" s="20" t="s">
         <v>263</v>
       </c>
-      <c r="C103" s="20">
+      <c r="C104" s="20">
         <v>1</v>
       </c>
-      <c r="D103" s="20" t="s">
+      <c r="D104" s="20" t="s">
         <v>135</v>
       </c>
-      <c r="E103" t="s">
+      <c r="E104" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A104" t="s">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
         <v>270</v>
       </c>
-      <c r="B104" s="31" t="s">
+      <c r="B105" s="30" t="s">
         <v>263</v>
       </c>
-      <c r="C104" s="31">
+      <c r="C105" s="30">
         <v>35000</v>
       </c>
-      <c r="D104" s="20" t="s">
+      <c r="D105" s="20" t="s">
         <v>271</v>
       </c>
-      <c r="E104" t="s">
+      <c r="E105" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A105" t="s">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
         <v>303</v>
       </c>
-      <c r="B105" s="27" t="s">
+      <c r="B106" s="27" t="s">
         <v>263</v>
       </c>
-      <c r="C105" s="27">
+      <c r="C106" s="27">
         <v>0.34599999999999997</v>
       </c>
-      <c r="D105" s="20" t="s">
+      <c r="D106" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="E105" t="s">
+      <c r="E106" t="s">
         <v>304</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A106" t="s">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
         <v>305</v>
       </c>
-      <c r="B106" s="20" t="s">
+      <c r="B107" s="20" t="s">
         <v>134</v>
       </c>
-      <c r="C106" s="20">
+      <c r="C107" s="20">
         <v>1000</v>
-      </c>
-      <c r="D106" s="20" t="s">
-        <v>309</v>
-      </c>
-      <c r="E106" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A107" t="s">
-        <v>306</v>
-      </c>
-      <c r="B107" s="20" t="s">
-        <v>168</v>
-      </c>
-      <c r="C107" s="20">
-        <v>890</v>
       </c>
       <c r="D107" s="20" t="s">
         <v>309</v>
       </c>
       <c r="E107" t="s">
-        <v>499</v>
-      </c>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.3">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="B108" s="20" t="s">
         <v>168</v>
       </c>
       <c r="C108" s="20">
-        <v>60</v>
+        <v>890</v>
       </c>
       <c r="D108" s="20" t="s">
-        <v>182</v>
+        <v>309</v>
       </c>
       <c r="E108" t="s">
         <v>499</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
+        <v>307</v>
+      </c>
+      <c r="B109" s="20" t="s">
+        <v>168</v>
+      </c>
+      <c r="C109" s="20">
+        <v>60</v>
+      </c>
+      <c r="D109" s="20" t="s">
+        <v>182</v>
+      </c>
+      <c r="E109" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
         <v>308</v>
       </c>
-      <c r="B109" s="20" t="s">
+      <c r="B110" s="20" t="s">
         <v>134</v>
       </c>
-      <c r="C109" s="20">
+      <c r="C110" s="20">
         <v>11.941543440928031</v>
       </c>
-      <c r="D109" s="20" t="s">
+      <c r="D110" s="20" t="s">
         <v>135</v>
       </c>
-      <c r="E109" t="s">
+      <c r="E110" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A110" s="22" t="s">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A111" s="22" t="s">
         <v>501</v>
-      </c>
-      <c r="B110" s="23" t="s">
-        <v>502</v>
-      </c>
-      <c r="C110" s="23">
-        <v>241</v>
-      </c>
-      <c r="D110" s="23" t="s">
-        <v>503</v>
-      </c>
-      <c r="E110" s="24" t="s">
-        <v>525</v>
-      </c>
-    </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A111" s="22" t="s">
-        <v>504</v>
       </c>
       <c r="B111" s="23" t="s">
         <v>502</v>
       </c>
-      <c r="C111" s="29">
-        <v>186</v>
+      <c r="C111" s="23">
+        <v>241</v>
       </c>
       <c r="D111" s="23" t="s">
         <v>503</v>
       </c>
-      <c r="E111" s="22" t="s">
+      <c r="E111" s="24" t="s">
         <v>525</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A112" s="22" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B112" s="23" t="s">
         <v>502</v>
       </c>
-      <c r="C112" s="23">
-        <v>462</v>
+      <c r="C112" s="29">
+        <v>186</v>
       </c>
       <c r="D112" s="23" t="s">
         <v>503</v>
       </c>
-      <c r="E112" s="24" t="s">
+      <c r="E112" s="22" t="s">
         <v>525</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A113" s="22" t="s">
-        <v>527</v>
+        <v>505</v>
       </c>
       <c r="B113" s="23" t="s">
         <v>502</v>
       </c>
       <c r="C113" s="23">
-        <v>30</v>
+        <v>462</v>
       </c>
       <c r="D113" s="23" t="s">
         <v>503</v>
       </c>
-      <c r="E113" s="22" t="s">
+      <c r="E113" s="24" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A114" s="22" t="s">
+        <v>527</v>
+      </c>
+      <c r="B114" s="23" t="s">
+        <v>502</v>
+      </c>
+      <c r="C114" s="23">
+        <v>30</v>
+      </c>
+      <c r="D114" s="23" t="s">
+        <v>503</v>
+      </c>
+      <c r="E114" s="22" t="s">
         <v>539</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A114" s="24" t="s">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A115" s="24" t="s">
         <v>559</v>
       </c>
-      <c r="B114" s="25" t="s">
+      <c r="B115" s="25" t="s">
         <v>502</v>
       </c>
-      <c r="C114" s="25">
+      <c r="C115" s="25">
         <v>9.5</v>
       </c>
-      <c r="D114" s="25" t="s">
+      <c r="D115" s="25" t="s">
         <v>503</v>
       </c>
-      <c r="E114" s="24" t="s">
+      <c r="E115" s="24" t="s">
         <v>539</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A115" s="22" t="s">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A116" s="22" t="s">
         <v>560</v>
-      </c>
-      <c r="B115" s="23" t="s">
-        <v>502</v>
-      </c>
-      <c r="C115" s="23">
-        <v>2.5</v>
-      </c>
-      <c r="D115" s="23" t="s">
-        <v>503</v>
-      </c>
-      <c r="E115" s="22" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A116" s="22" t="s">
-        <v>506</v>
       </c>
       <c r="B116" s="23" t="s">
         <v>502</v>
       </c>
-      <c r="C116" s="26">
-        <v>68900</v>
+      <c r="C116" s="23">
+        <v>2.5</v>
       </c>
       <c r="D116" s="23" t="s">
         <v>503</v>
       </c>
-      <c r="E116" s="24" t="s">
+      <c r="E116" s="22" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A117" s="22" t="s">
+        <v>506</v>
+      </c>
+      <c r="B117" s="23" t="s">
+        <v>502</v>
+      </c>
+      <c r="C117" s="26">
+        <v>68900</v>
+      </c>
+      <c r="D117" s="23" t="s">
+        <v>503</v>
+      </c>
+      <c r="E117" s="24" t="s">
         <v>526</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A117" s="22" t="s">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A118" s="22" t="s">
         <v>522</v>
-      </c>
-      <c r="B117" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="C117" s="23">
-        <v>0.14799999999999999</v>
-      </c>
-      <c r="D117" s="23" t="s">
-        <v>59</v>
-      </c>
-      <c r="E117" s="22" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A118" s="22" t="s">
-        <v>507</v>
       </c>
       <c r="B118" s="23" t="s">
         <v>56</v>
       </c>
       <c r="C118" s="23">
-        <v>4.0000000000000001E-3</v>
+        <v>0.14799999999999999</v>
       </c>
       <c r="D118" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="E118" s="24"/>
-    </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E118" s="22" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A119" s="22" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B119" s="23" t="s">
         <v>56</v>
       </c>
       <c r="C119" s="23">
-        <v>0.04</v>
+        <v>4.0000000000000001E-3</v>
       </c>
       <c r="D119" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="E119" s="22"/>
-    </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E119" s="24"/>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A120" s="22" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="B120" s="23" t="s">
         <v>56</v>
       </c>
       <c r="C120" s="23">
-        <v>2.3E-2</v>
+        <v>0.04</v>
       </c>
       <c r="D120" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="E120" s="24"/>
-    </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E120" s="22"/>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A121" s="22" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="B121" s="23" t="s">
         <v>56</v>
       </c>
       <c r="C121" s="23">
-        <v>50</v>
+        <v>2.3E-2</v>
       </c>
       <c r="D121" s="23" t="s">
-        <v>23</v>
-      </c>
-      <c r="E121" s="22"/>
-    </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+      <c r="E121" s="24"/>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A122" s="22" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B122" s="23" t="s">
         <v>56</v>
       </c>
       <c r="C122" s="23">
-        <v>0.09</v>
+        <v>50</v>
       </c>
       <c r="D122" s="23" t="s">
-        <v>59</v>
-      </c>
-      <c r="E122" s="24"/>
-    </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+      <c r="E122" s="22"/>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A123" s="22" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="B123" s="23" t="s">
         <v>56</v>
       </c>
       <c r="C123" s="23">
-        <v>6.3499999999999997E-3</v>
+        <v>0.09</v>
       </c>
       <c r="D123" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="E123" s="22"/>
-    </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E123" s="24"/>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A124" s="22" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="B124" s="23" t="s">
         <v>56</v>
       </c>
       <c r="C124" s="23">
-        <v>1.2699999999999999E-2</v>
+        <v>6.3499999999999997E-3</v>
       </c>
       <c r="D124" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="E124" s="24"/>
-    </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E124" s="22"/>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A125" s="22" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="B125" s="23" t="s">
         <v>56</v>
       </c>
       <c r="C125" s="23">
-        <v>0.76</v>
+        <v>1.2699999999999999E-2</v>
       </c>
       <c r="D125" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="E125" s="22"/>
-    </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E125" s="24"/>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A126" s="22" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B126" s="23" t="s">
         <v>56</v>
       </c>
       <c r="C126" s="23">
-        <v>1.524E-3</v>
+        <v>0.76</v>
       </c>
       <c r="D126" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="E126" s="24"/>
-    </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E126" s="22"/>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A127" s="22" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="B127" s="23" t="s">
         <v>56</v>
       </c>
       <c r="C127" s="23">
-        <v>1.2699999999999999E-2</v>
+        <v>1.524E-3</v>
       </c>
       <c r="D127" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="E127" s="22"/>
-    </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E127" s="24"/>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A128" s="22" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B128" s="23" t="s">
         <v>56</v>
       </c>
       <c r="C128" s="23">
-        <v>0.56499999999999995</v>
+        <v>1.2699999999999999E-2</v>
       </c>
       <c r="D128" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="E128" s="24" t="s">
-        <v>561</v>
-      </c>
-    </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E128" s="22"/>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A129" s="22" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="B129" s="23" t="s">
         <v>56</v>
       </c>
       <c r="C129" s="23">
-        <v>1.524E-3</v>
+        <v>0.56499999999999995</v>
       </c>
       <c r="D129" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="E129" s="22"/>
-    </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E129" s="24" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A130" s="22" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B130" s="23" t="s">
         <v>56</v>
       </c>
       <c r="C130" s="23">
-        <v>8.9999999999999993E-3</v>
+        <v>1.524E-3</v>
       </c>
       <c r="D130" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="E130" s="24"/>
-    </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E130" s="22"/>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A131" s="22" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="B131" s="23" t="s">
         <v>56</v>
       </c>
       <c r="C131" s="23">
-        <v>4.3E-3</v>
+        <v>8.9999999999999993E-3</v>
       </c>
       <c r="D131" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="E131" s="22"/>
-    </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A132" s="24" t="s">
+      <c r="E131" s="24"/>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A132" s="22" t="s">
+        <v>520</v>
+      </c>
+      <c r="B132" s="23" t="s">
+        <v>56</v>
+      </c>
+      <c r="C132" s="23">
+        <v>4.3E-3</v>
+      </c>
+      <c r="D132" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="E132" s="22"/>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A133" s="24" t="s">
         <v>562</v>
       </c>
-      <c r="B132" s="25" t="s">
+      <c r="B133" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="C132" s="25">
+      <c r="C133" s="25">
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="D132" s="25" t="s">
+      <c r="D133" s="25" t="s">
         <v>59</v>
       </c>
-      <c r="E132" s="24"/>
+      <c r="E133" s="24"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4478,18 +4493,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H168"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.6640625" customWidth="1"/>
-    <col min="2" max="2" width="12.5546875" customWidth="1"/>
-    <col min="3" max="3" width="64.5546875" customWidth="1"/>
-    <col min="4" max="4" width="5.6640625" customWidth="1"/>
+    <col min="1" max="1" width="40.7109375" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" customWidth="1"/>
+    <col min="3" max="3" width="64.5703125" customWidth="1"/>
+    <col min="4" max="4" width="5.7109375" customWidth="1"/>
     <col min="5" max="5" width="46" customWidth="1"/>
-    <col min="6" max="6" width="32.44140625" customWidth="1"/>
-    <col min="8" max="8" width="42.6640625" customWidth="1"/>
+    <col min="6" max="6" width="32.42578125" customWidth="1"/>
+    <col min="8" max="8" width="42.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4512,7 +4527,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>313</v>
       </c>
@@ -4532,7 +4547,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>314</v>
       </c>
@@ -4552,7 +4567,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>315</v>
       </c>
@@ -4572,7 +4587,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>316</v>
       </c>
@@ -4592,7 +4607,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>317</v>
       </c>
@@ -4612,7 +4627,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>318</v>
       </c>
@@ -4626,7 +4641,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>319</v>
       </c>
@@ -4646,7 +4661,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>320</v>
       </c>
@@ -4666,7 +4681,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>321</v>
       </c>
@@ -4686,7 +4701,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>322</v>
       </c>
@@ -4706,7 +4721,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>323</v>
       </c>
@@ -4726,7 +4741,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>378</v>
       </c>
@@ -4740,7 +4755,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>379</v>
       </c>
@@ -4754,7 +4769,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>380</v>
       </c>
@@ -4768,7 +4783,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>381</v>
       </c>
@@ -4782,7 +4797,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>382</v>
       </c>
@@ -4796,7 +4811,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>383</v>
       </c>
@@ -4810,7 +4825,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>384</v>
       </c>
@@ -4824,7 +4839,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>385</v>
       </c>
@@ -4838,7 +4853,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>386</v>
       </c>
@@ -4852,7 +4867,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>387</v>
       </c>
@@ -4866,7 +4881,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>500</v>
       </c>
@@ -4880,7 +4895,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>324</v>
       </c>
@@ -4900,7 +4915,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>325</v>
       </c>
@@ -4920,7 +4935,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>326</v>
       </c>
@@ -4940,7 +4955,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>327</v>
       </c>
@@ -4960,7 +4975,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>328</v>
       </c>
@@ -4980,7 +4995,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>329</v>
       </c>
@@ -5000,7 +5015,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>330</v>
       </c>
@@ -5020,7 +5035,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>331</v>
       </c>
@@ -5040,7 +5055,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>332</v>
       </c>
@@ -5060,7 +5075,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>333</v>
       </c>
@@ -5080,7 +5095,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>334</v>
       </c>
@@ -5100,7 +5115,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>388</v>
       </c>
@@ -5114,7 +5129,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>389</v>
       </c>
@@ -5128,7 +5143,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>390</v>
       </c>
@@ -5142,7 +5157,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>391</v>
       </c>
@@ -5156,7 +5171,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>165</v>
       </c>
@@ -5170,7 +5185,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>335</v>
       </c>
@@ -5190,7 +5205,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>336</v>
       </c>
@@ -5210,7 +5225,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>337</v>
       </c>
@@ -5230,7 +5245,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>338</v>
       </c>
@@ -5250,7 +5265,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>339</v>
       </c>
@@ -5270,7 +5285,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>340</v>
       </c>
@@ -5290,7 +5305,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>341</v>
       </c>
@@ -5310,7 +5325,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>342</v>
       </c>
@@ -5324,7 +5339,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>343</v>
       </c>
@@ -5338,7 +5353,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>344</v>
       </c>
@@ -5352,7 +5367,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>392</v>
       </c>
@@ -5366,7 +5381,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>528</v>
       </c>
@@ -5380,7 +5395,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>393</v>
       </c>
@@ -5394,7 +5409,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>403</v>
       </c>
@@ -5408,7 +5423,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>404</v>
       </c>
@@ -5422,7 +5437,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>405</v>
       </c>
@@ -5436,7 +5451,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>406</v>
       </c>
@@ -5450,7 +5465,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>407</v>
       </c>
@@ -5464,7 +5479,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>394</v>
       </c>
@@ -5478,7 +5493,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>395</v>
       </c>
@@ -5492,7 +5507,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>396</v>
       </c>
@@ -5506,7 +5521,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>397</v>
       </c>
@@ -5520,7 +5535,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>398</v>
       </c>
@@ -5534,7 +5549,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>399</v>
       </c>
@@ -5548,7 +5563,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>400</v>
       </c>
@@ -5562,7 +5577,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>401</v>
       </c>
@@ -5576,7 +5591,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>402</v>
       </c>
@@ -5590,7 +5605,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>408</v>
       </c>
@@ -5604,7 +5619,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>409</v>
       </c>
@@ -5618,7 +5633,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>410</v>
       </c>
@@ -5632,7 +5647,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>411</v>
       </c>
@@ -5646,7 +5661,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>412</v>
       </c>
@@ -5660,7 +5675,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>413</v>
       </c>
@@ -5674,7 +5689,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>414</v>
       </c>
@@ -5688,7 +5703,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>415</v>
       </c>
@@ -5702,7 +5717,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>416</v>
       </c>
@@ -5716,7 +5731,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>417</v>
       </c>
@@ -5730,7 +5745,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>418</v>
       </c>
@@ -5744,7 +5759,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>419</v>
       </c>
@@ -5758,7 +5773,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>420</v>
       </c>
@@ -5772,7 +5787,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>421</v>
       </c>
@@ -5786,7 +5801,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>422</v>
       </c>
@@ -5800,7 +5815,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>423</v>
       </c>
@@ -5814,7 +5829,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>424</v>
       </c>
@@ -5828,7 +5843,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>425</v>
       </c>
@@ -5842,7 +5857,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>426</v>
       </c>
@@ -5856,7 +5871,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>427</v>
       </c>
@@ -5870,7 +5885,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>428</v>
       </c>
@@ -5884,7 +5899,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>429</v>
       </c>
@@ -5898,7 +5913,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>430</v>
       </c>
@@ -5912,7 +5927,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>431</v>
       </c>
@@ -5926,7 +5941,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>432</v>
       </c>
@@ -5940,7 +5955,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>433</v>
       </c>
@@ -5954,7 +5969,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>434</v>
       </c>
@@ -5968,7 +5983,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>435</v>
       </c>
@@ -5982,7 +5997,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>436</v>
       </c>
@@ -5996,7 +6011,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>437</v>
       </c>
@@ -6010,7 +6025,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>438</v>
       </c>
@@ -6024,7 +6039,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>439</v>
       </c>
@@ -6038,7 +6053,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>440</v>
       </c>
@@ -6052,7 +6067,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>441</v>
       </c>
@@ -6066,7 +6081,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>442</v>
       </c>
@@ -6080,7 +6095,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>443</v>
       </c>
@@ -6094,7 +6109,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>444</v>
       </c>
@@ -6108,7 +6123,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>445</v>
       </c>
@@ -6122,7 +6137,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>446</v>
       </c>
@@ -6136,7 +6151,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>447</v>
       </c>
@@ -6150,7 +6165,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>529</v>
       </c>
@@ -6164,7 +6179,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>448</v>
       </c>
@@ -6178,7 +6193,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>449</v>
       </c>
@@ -6192,7 +6207,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>450</v>
       </c>
@@ -6206,7 +6221,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>451</v>
       </c>
@@ -6220,7 +6235,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>452</v>
       </c>
@@ -6234,7 +6249,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>453</v>
       </c>
@@ -6248,7 +6263,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>454</v>
       </c>
@@ -6262,7 +6277,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>455</v>
       </c>
@@ -6276,7 +6291,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>456</v>
       </c>
@@ -6290,7 +6305,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>457</v>
       </c>
@@ -6304,7 +6319,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>458</v>
       </c>
@@ -6318,7 +6333,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>459</v>
       </c>
@@ -6332,7 +6347,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>460</v>
       </c>
@@ -6346,7 +6361,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>461</v>
       </c>
@@ -6360,7 +6375,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>462</v>
       </c>
@@ -6374,7 +6389,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>540</v>
       </c>
@@ -6388,7 +6403,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>541</v>
       </c>
@@ -6402,7 +6417,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>542</v>
       </c>
@@ -6416,7 +6431,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>543</v>
       </c>
@@ -6430,7 +6445,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>544</v>
       </c>
@@ -6444,7 +6459,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>530</v>
       </c>
@@ -6458,7 +6473,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>531</v>
       </c>
@@ -6472,7 +6487,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>545</v>
       </c>
@@ -6486,7 +6501,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>546</v>
       </c>
@@ -6500,7 +6515,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>547</v>
       </c>
@@ -6514,7 +6529,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>548</v>
       </c>
@@ -6528,7 +6543,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>549</v>
       </c>
@@ -6542,7 +6557,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>532</v>
       </c>
@@ -6556,7 +6571,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>533</v>
       </c>
@@ -6570,7 +6585,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>550</v>
       </c>
@@ -6584,7 +6599,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>551</v>
       </c>
@@ -6598,7 +6613,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>552</v>
       </c>
@@ -6612,7 +6627,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>553</v>
       </c>
@@ -6626,7 +6641,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>534</v>
       </c>
@@ -6640,7 +6655,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>535</v>
       </c>
@@ -6654,7 +6669,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>554</v>
       </c>
@@ -6668,7 +6683,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>555</v>
       </c>
@@ -6682,7 +6697,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>556</v>
       </c>
@@ -6696,7 +6711,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>557</v>
       </c>
@@ -6710,7 +6725,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>536</v>
       </c>
@@ -6724,7 +6739,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>537</v>
       </c>
@@ -6738,7 +6753,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>463</v>
       </c>
@@ -6752,7 +6767,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>464</v>
       </c>
@@ -6766,7 +6781,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>465</v>
       </c>
@@ -6780,7 +6795,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>466</v>
       </c>
@@ -6794,7 +6809,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>467</v>
       </c>
@@ -6808,7 +6823,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>468</v>
       </c>
@@ -6822,7 +6837,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>469</v>
       </c>
@@ -6836,7 +6851,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>470</v>
       </c>
@@ -6850,7 +6865,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>471</v>
       </c>
@@ -6864,7 +6879,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>472</v>
       </c>
@@ -6878,7 +6893,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>473</v>
       </c>
@@ -6892,7 +6907,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>474</v>
       </c>
@@ -6906,7 +6921,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>475</v>
       </c>
@@ -6920,7 +6935,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>476</v>
       </c>
@@ -6934,7 +6949,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>477</v>
       </c>
@@ -6948,7 +6963,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>478</v>
       </c>
@@ -6962,7 +6977,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>479</v>
       </c>
@@ -6976,7 +6991,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>480</v>
       </c>
@@ -6990,7 +7005,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>481</v>
       </c>
@@ -7004,7 +7019,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>482</v>
       </c>
@@ -7026,14 +7041,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFCC8514-E0AF-4C67-BF86-8649FC702924}">
   <dimension ref="A1:D20"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="32.44140625" customWidth="1"/>
-    <col min="2" max="3" width="32.44140625" style="20" customWidth="1"/>
-    <col min="4" max="4" width="13.33203125" style="20" customWidth="1"/>
+    <col min="1" max="1" width="32.42578125" customWidth="1"/>
+    <col min="2" max="3" width="32.42578125" style="20" customWidth="1"/>
+    <col min="4" max="4" width="13.28515625" style="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
         <v>272</v>
       </c>
@@ -7047,7 +7062,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>274</v>
       </c>
@@ -7061,7 +7076,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="21" t="s">
         <v>275</v>
       </c>
@@ -7075,7 +7090,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>276</v>
       </c>
@@ -7089,7 +7104,7 @@
         <v>5.6000000000000001E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>277</v>
       </c>
@@ -7103,7 +7118,7 @@
         <v>1.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="21" t="s">
         <v>302</v>
       </c>
@@ -7117,7 +7132,7 @@
         <v>-2.1999999999999999E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>278</v>
       </c>
@@ -7131,7 +7146,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>279</v>
       </c>
@@ -7145,7 +7160,7 @@
         <v>5.2999999999999999E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>280</v>
       </c>
@@ -7159,7 +7174,7 @@
         <v>8.6999999999999994E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>281</v>
       </c>
@@ -7173,7 +7188,7 @@
         <v>0.125</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>282</v>
       </c>
@@ -7187,7 +7202,7 @@
         <v>0.14599999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>283</v>
       </c>
@@ -7201,7 +7216,7 @@
         <v>0.14599999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>284</v>
       </c>
@@ -7215,7 +7230,7 @@
         <v>3.2000000000000001E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>285</v>
       </c>
@@ -7229,7 +7244,7 @@
         <v>0.126</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
         <v>286</v>
       </c>
@@ -7243,7 +7258,7 @@
         <v>-4.3999999999999997E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>287</v>
       </c>
@@ -7257,7 +7272,7 @@
         <v>4.5999999999999999E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>288</v>
       </c>
@@ -7271,7 +7286,7 @@
         <v>0.11700000000000001</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>289</v>
       </c>
@@ -7285,7 +7300,7 @@
         <v>7.2999999999999995E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>291</v>
       </c>
@@ -7299,7 +7314,7 @@
         <v>7.6999999999999999E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>290</v>
       </c>
@@ -7321,26 +7336,26 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{118BE621-EF6B-4648-868E-9937B9C5B685}">
   <dimension ref="A1:F32"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="48.109375" style="2" customWidth="1"/>
-    <col min="2" max="4" width="15.6640625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="3.6640625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="46.6640625" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="8.6640625" style="2"/>
+    <col min="1" max="1" width="48.140625" style="2" customWidth="1"/>
+    <col min="2" max="4" width="15.7109375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="3.7109375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="46.7109375" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="8.7109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>206</v>
       </c>
@@ -7354,7 +7369,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>210</v>
       </c>
@@ -7372,7 +7387,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>212</v>
       </c>
@@ -7392,7 +7407,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>214</v>
       </c>
@@ -7412,7 +7427,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>215</v>
       </c>
@@ -7430,7 +7445,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>216</v>
       </c>
@@ -7450,7 +7465,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>218</v>
       </c>
@@ -7467,7 +7482,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>220</v>
       </c>
@@ -7484,7 +7499,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>221</v>
       </c>
@@ -7504,7 +7519,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>223</v>
       </c>
@@ -7521,47 +7536,47 @@
         <v>224</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>255</v>
       </c>
       <c r="B14" s="17">
-        <f>Inputs!C91</f>
+        <f>Inputs!C92</f>
         <v>1</v>
       </c>
       <c r="C14" s="17">
-        <f>Inputs!C92</f>
+        <f>Inputs!C93</f>
         <v>1.2</v>
       </c>
       <c r="D14" s="17">
-        <f>Inputs!C93</f>
+        <f>Inputs!C94</f>
         <v>1</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>257</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>256</v>
       </c>
       <c r="B15" s="17">
-        <f>Inputs!C94</f>
+        <f>Inputs!C95</f>
         <v>0.85</v>
       </c>
       <c r="C15" s="17">
-        <f>Inputs!C94</f>
+        <f>Inputs!C95</f>
         <v>0.85</v>
       </c>
       <c r="D15" s="17">
-        <f>Inputs!C94</f>
+        <f>Inputs!C95</f>
         <v>0.85</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>258</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>225</v>
       </c>
@@ -7569,7 +7584,7 @@
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>226</v>
       </c>
@@ -7586,7 +7601,7 @@
         <v>1.9823131728623846</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>227</v>
       </c>
@@ -7603,7 +7618,7 @@
         <v>1.1592794807274085</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>228</v>
       </c>
@@ -7620,7 +7635,7 @@
         <v>-0.62740704594148844</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>229</v>
       </c>
@@ -7637,7 +7652,7 @@
         <v>-0.96540266006846076</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>230</v>
       </c>
@@ -7645,7 +7660,7 @@
       <c r="C21" s="4"/>
       <c r="D21" s="4"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>231</v>
       </c>
@@ -7662,7 +7677,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>232</v>
       </c>
@@ -7679,7 +7694,7 @@
         <v>0.52359877559829882</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>233</v>
       </c>
@@ -7696,7 +7711,7 @@
         <v>-0.50548365077118673</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>234</v>
       </c>
@@ -7713,7 +7728,7 @@
         <v>324.01250000000005</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>235</v>
       </c>
@@ -7730,7 +7745,7 @@
         <v>1.42884E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
         <v>236</v>
       </c>
@@ -7747,7 +7762,7 @@
         <v>-0.13760360258695806</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>237</v>
       </c>
@@ -7764,7 +7779,7 @@
         <v>0.13760360258695806</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
         <v>238</v>
       </c>
@@ -7781,7 +7796,7 @@
         <v>22.925083964169769</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
         <v>239</v>
       </c>
@@ -7789,7 +7804,7 @@
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>240</v>
       </c>
@@ -7797,7 +7812,7 @@
       <c r="C31" s="14"/>
       <c r="D31" s="14"/>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>241</v>
       </c>
@@ -7822,13 +7837,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="C109:F109"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="11.5546875" customWidth="1"/>
-    <col min="6" max="6" width="142.44140625" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" customWidth="1"/>
+    <col min="6" max="6" width="142.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="109" spans="3:6" x14ac:dyDescent="0.3">
+    <row r="109" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C109">
         <v>11.941543440928031</v>
       </c>

</xml_diff>

<commit_message>
margin I hardly know her
</commit_message>
<xml_diff>
--- a/SizingParams.xlsx
+++ b/SizingParams.xlsx
@@ -1617,7 +1617,7 @@
     <t>From UltiMaker</t>
   </si>
   <si>
-    <t>Written by writeOutputs.m on 2026-10-08 15:10</t>
+    <t>Written by writeOutputs.m on 2026-10-08 15:49</t>
   </si>
 </sst>
 </file>
@@ -6291,7 +6291,7 @@
         <v>263</v>
       </c>
       <c r="C120">
-        <v>13.049693149492025</v>
+        <v>0.92725557606200626</v>
       </c>
       <c r="F120" t="s">
         <v>375</v>

</xml_diff>

<commit_message>
update XFLR with MOIs
</commit_message>
<xml_diff>
--- a/SizingParams.xlsx
+++ b/SizingParams.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="libxl" lastEdited="7" lowestEdited="7" rupBuild="5000000"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E190E2B-2CFE-4A75-8856-7C36167B196A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="Hinge Moments" sheetId="2" r:id="rId4"/>
     <sheet name="Sheet1" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="true"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1081" uniqueCount="527">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="1564" uniqueCount="528">
   <si>
     <t>Parameter</t>
   </si>
@@ -1618,18 +1618,21 @@
   </si>
   <si>
     <t>Written by writeOutputs.m on 2026-10-08 15:49</t>
+  </si>
+  <si>
+    <t>Written by writeOutputs.m on 2026-10-15 10:53</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1725,8 +1728,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
-        <bgColor theme="0" tint="-0.14999847407452621"/>
+        <fgColor theme="0" tint="-0.14999847407453"/>
+        <bgColor theme="0" tint="-0.14999847407453"/>
       </patternFill>
     </fill>
     <fill>
@@ -1737,12 +1740,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <fgColor theme="0" tint="-0.14999847407453"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1765,75 +1768,77 @@
       </bottom>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="false" applyFill="false" applyBorder="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="true"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="5" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="6" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="5" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="5" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="true"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="true" applyFill="true"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="true"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="true"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="true"/>
+    <xf numFmtId="166" fontId="5" fillId="3" borderId="0" xfId="1" applyNumberFormat="true" applyFont="true" applyFill="true"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="1" applyNumberFormat="true" applyFont="true" applyFill="true"/>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="0" xfId="1" applyNumberFormat="true" applyFont="true" applyFill="true"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="true"/>
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="0" xfId="1" applyNumberFormat="true" applyFont="true" applyFill="true"/>
+    <xf numFmtId="2" fontId="6" fillId="4" borderId="0" xfId="1" applyNumberFormat="true" applyFont="true" applyFill="true"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="1" applyFont="true" applyFill="true"/>
+    <xf numFmtId="164" fontId="1" fillId="3" borderId="0" xfId="1" applyNumberFormat="true" applyFill="true"/>
+    <xf numFmtId="166" fontId="5" fillId="5" borderId="0" xfId="1" applyNumberFormat="true" applyFont="true" applyFill="true"/>
+    <xf numFmtId="2" fontId="5" fillId="5" borderId="0" xfId="1" applyNumberFormat="true" applyFont="true" applyFill="true"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="true" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="11" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="11" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="true" applyAlignment="true">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
   <dxfs count="3">
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" justifyLastLine="false" shrinkToFit="false" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" justifyLastLine="false" shrinkToFit="false" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" justifyLastLine="false" shrinkToFit="false" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1849,25 +1854,25 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:F148" totalsRowShown="0">
-  <autoFilter ref="A1:F148" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E43">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" id="1" name="Table1" displayName="Table1" ref="A1:F148" totalsRowShown="false">
+  <autoFilter ref="A1:F148"/>
+  <sortState ref="A2:E43">
     <sortCondition ref="B1:B102"/>
   </sortState>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Parameter"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Subclass" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Value" dataDxfId="1"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Units" dataDxfId="0"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Description"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Notes"/>
+    <tableColumn id="1" name="Parameter"/>
+    <tableColumn id="2" name="Subclass" dataDxfId="2"/>
+    <tableColumn id="3" name="Value" dataDxfId="1"/>
+    <tableColumn id="4" name="Units" dataDxfId="0"/>
+    <tableColumn id="5" name="Description"/>
+    <tableColumn id="6" name="Notes"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium15" showFirstColumn="false" showLastColumn="false" showRowStripes="true" showColumnStripes="false"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1984,7 +1989,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -2008,9 +2013,9 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -2034,7 +2039,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -2069,7 +2074,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="false">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -2087,7 +2092,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -2112,7 +2117,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
@@ -4427,2155 +4432,2657 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H140"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.7109375" customWidth="1"/>
-    <col min="2" max="2" width="12.5703125" customWidth="1"/>
-    <col min="3" max="3" width="33.42578125" customWidth="1"/>
-    <col min="4" max="4" width="5.7109375" customWidth="1"/>
-    <col min="5" max="5" width="46" customWidth="1"/>
-    <col min="6" max="6" width="32.42578125" customWidth="1"/>
-    <col min="8" max="8" width="42.7109375" customWidth="1"/>
+    <col min="1" max="1" width="40.7109375" customWidth="true"/>
+    <col min="2" max="2" width="12.5703125" customWidth="true"/>
+    <col min="3" max="3" width="33.42578125" customWidth="true"/>
+    <col min="4" max="4" width="5.7109375" customWidth="true"/>
+    <col min="5" max="5" width="46" customWidth="true"/>
+    <col min="6" max="6" width="32.42578125" customWidth="true"/>
+    <col min="8" max="8" width="42.7109375" customWidth="true"/>
+    <col min="7" max="7" width="9.140625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1">
+      <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="0" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="0" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="0" t="s">
         <v>374</v>
       </c>
-      <c r="H1" t="s">
-        <v>526</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="G1" s="0"/>
+      <c r="H1" s="0" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="s">
         <v>313</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="C2">
-        <v>0.3</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="C2" s="0">
+        <v>0.29999999999999999</v>
+      </c>
+      <c r="D2" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="0" t="s">
         <v>346</v>
       </c>
-      <c r="F2" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="F2" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G2" s="0"/>
+      <c r="H2" s="0"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="s">
         <v>314</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="0">
         <v>1.1818181818181817</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="0" t="s">
         <v>347</v>
       </c>
-      <c r="F3" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="F3" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G3" s="0"/>
+      <c r="H3" s="0"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="s">
         <v>315</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="0">
         <v>0.92582241145109656</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="0" t="s">
         <v>348</v>
       </c>
-      <c r="F4" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="F4" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G4" s="0"/>
+      <c r="H4" s="0"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="s">
         <v>316</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="C5">
-        <v>8.0941856394028303E-2</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="C5" s="0">
+        <v>0.080941856394028303</v>
+      </c>
+      <c r="D5" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="0" t="s">
         <v>349</v>
       </c>
-      <c r="F5" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="F5" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G5" s="0"/>
+      <c r="H5" s="0"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="s">
         <v>317</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="0">
         <v>0.19588300688233271</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="0" t="s">
         <v>350</v>
       </c>
-      <c r="F6" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="F6" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G6" s="0"/>
+      <c r="H6" s="0"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="s">
         <v>318</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="C7">
-        <v>3.1335225950127228E-2</v>
-      </c>
-      <c r="F7" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="C7" s="0">
+        <v>0.031335225950127228</v>
+      </c>
+      <c r="D7" s="0"/>
+      <c r="E7" s="0"/>
+      <c r="F7" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G7" s="0"/>
+      <c r="H7" s="0"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="s">
         <v>319</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="C8">
-        <v>3.8619993025589772E-2</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="C8" s="0">
+        <v>0.038619993025589772</v>
+      </c>
+      <c r="D8" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="0" t="s">
         <v>351</v>
       </c>
-      <c r="F8" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="F8" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G8" s="0"/>
+      <c r="H8" s="0"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="s">
         <v>320</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="C9">
-        <v>3.8619993025589772E-2</v>
-      </c>
-      <c r="D9" t="s">
+      <c r="C9" s="0">
+        <v>0.038619993025589772</v>
+      </c>
+      <c r="D9" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="0" t="s">
         <v>352</v>
       </c>
-      <c r="F9" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="F9" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G9" s="0"/>
+      <c r="H9" s="0"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="s">
         <v>321</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="C10">
-        <v>2.3619993025589772E-2</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="C10" s="0">
+        <v>0.023619993025589772</v>
+      </c>
+      <c r="D10" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="0" t="s">
         <v>353</v>
       </c>
-      <c r="F10" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="F10" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G10" s="0"/>
+      <c r="H10" s="0"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="s">
         <v>322</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="C11">
+      <c r="C11" s="0">
         <v>7.7679972598964149</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="0" t="s">
         <v>354</v>
       </c>
-      <c r="F11" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="F11" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G11" s="0"/>
+      <c r="H11" s="0"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="s">
         <v>323</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="C12">
+      <c r="C12" s="0">
         <v>9.9281197918699284</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="0" t="s">
         <v>355</v>
       </c>
-      <c r="F12" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="F12" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G12" s="0"/>
+      <c r="H12" s="0"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="s">
         <v>378</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="C13">
+      <c r="C13" s="0">
         <v>3.0198549799930445</v>
       </c>
-      <c r="F13" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="D13" s="0"/>
+      <c r="E13" s="0"/>
+      <c r="F13" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G13" s="0"/>
+      <c r="H13" s="0"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="s">
         <v>379</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="C14">
+      <c r="C14" s="0">
         <v>3.9888876554460642</v>
       </c>
-      <c r="F14" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="D14" s="0"/>
+      <c r="E14" s="0"/>
+      <c r="F14" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G14" s="0"/>
+      <c r="H14" s="0"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="s">
         <v>380</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="0">
         <v>0.59783680842556775</v>
       </c>
-      <c r="F15" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="D15" s="0"/>
+      <c r="E15" s="0"/>
+      <c r="F15" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G15" s="0"/>
+      <c r="H15" s="0"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="s">
         <v>381</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="C16">
+      <c r="C16" s="0">
         <v>5.2033621722920103</v>
       </c>
-      <c r="F16" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="D16" s="0"/>
+      <c r="E16" s="0"/>
+      <c r="F16" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G16" s="0"/>
+      <c r="H16" s="0"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="s">
         <v>382</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="C17">
-        <v>-9.6561353939117869E-2</v>
-      </c>
-      <c r="F17" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="C17" s="0">
+        <v>-0.096561353939117869</v>
+      </c>
+      <c r="D17" s="0"/>
+      <c r="E17" s="0"/>
+      <c r="F17" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G17" s="0"/>
+      <c r="H17" s="0"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="s">
         <v>383</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="0">
         <v>0.66074594914354523</v>
       </c>
-      <c r="F18" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+      <c r="D18" s="0"/>
+      <c r="E18" s="0"/>
+      <c r="F18" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G18" s="0"/>
+      <c r="H18" s="0"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="s">
         <v>384</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="C19">
+      <c r="C19" s="0">
         <v>0.60899778104422941</v>
       </c>
-      <c r="F19" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+      <c r="D19" s="0"/>
+      <c r="E19" s="0"/>
+      <c r="F19" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G19" s="0"/>
+      <c r="H19" s="0"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="s">
         <v>385</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="C20">
+      <c r="C20" s="0">
         <v>1.5753270213496304</v>
       </c>
-      <c r="F20" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+      <c r="D20" s="0"/>
+      <c r="E20" s="0"/>
+      <c r="F20" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G20" s="0"/>
+      <c r="H20" s="0"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="s">
         <v>386</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="C21">
+      <c r="C21" s="0">
         <v>0.66074594914354523</v>
       </c>
-      <c r="F21" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+      <c r="D21" s="0"/>
+      <c r="E21" s="0"/>
+      <c r="F21" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G21" s="0"/>
+      <c r="H21" s="0"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="s">
         <v>387</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="C22">
+      <c r="C22" s="0">
         <v>0.12602616170797043</v>
       </c>
-      <c r="F22" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+      <c r="D22" s="0"/>
+      <c r="E22" s="0"/>
+      <c r="F22" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G22" s="0"/>
+      <c r="H22" s="0"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="s">
         <v>454</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="C23">
+      <c r="C23" s="0">
         <v>0.78050169904696809</v>
       </c>
-      <c r="F23" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+      <c r="D23" s="0"/>
+      <c r="E23" s="0"/>
+      <c r="F23" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G23" s="0"/>
+      <c r="H23" s="0"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="s">
         <v>324</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="0" t="s">
         <v>56</v>
       </c>
-      <c r="C24">
+      <c r="C24" s="0">
         <v>0.50145310681164035</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="0" t="s">
         <v>66</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E24" s="0" t="s">
         <v>356</v>
       </c>
-      <c r="F24" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+      <c r="F24" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G24" s="0"/>
+      <c r="H24" s="0"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="s">
         <v>325</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="0" t="s">
         <v>56</v>
       </c>
-      <c r="C25">
+      <c r="C25" s="0">
         <v>0.3531359907124228</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="0" t="s">
         <v>59</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E25" s="0" t="s">
         <v>357</v>
       </c>
-      <c r="F25" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+      <c r="F25" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G25" s="0"/>
+      <c r="H25" s="0"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="s">
         <v>326</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="0" t="s">
         <v>56</v>
       </c>
-      <c r="C26">
+      <c r="C26" s="0">
         <v>4.2476554059921039</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D26" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E26" s="0" t="s">
         <v>358</v>
       </c>
-      <c r="F26" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+      <c r="F26" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G26" s="0"/>
+      <c r="H26" s="0"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="s">
         <v>327</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="0" t="s">
         <v>56</v>
       </c>
-      <c r="C27">
-        <v>8.5247028157978869E-2</v>
-      </c>
-      <c r="D27" t="s">
+      <c r="C27" s="0">
+        <v>0.085247028157978869</v>
+      </c>
+      <c r="D27" s="0" t="s">
         <v>66</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E27" s="0" t="s">
         <v>359</v>
       </c>
-      <c r="F27" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+      <c r="F27" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G27" s="0"/>
+      <c r="H27" s="0"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="s">
         <v>328</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="0" t="s">
         <v>56</v>
       </c>
-      <c r="C28">
+      <c r="C28" s="0">
         <v>0.46164658603194192</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D28" s="0" t="s">
         <v>59</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E28" s="0" t="s">
         <v>360</v>
       </c>
-      <c r="F28" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+      <c r="F28" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G28" s="0"/>
+      <c r="H28" s="0"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="s">
         <v>329</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="0" t="s">
         <v>56</v>
       </c>
-      <c r="C29">
+      <c r="C29" s="0">
         <v>0.18465863441277677</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D29" s="0" t="s">
         <v>59</v>
       </c>
-      <c r="E29" t="s">
+      <c r="E29" s="0" t="s">
         <v>361</v>
       </c>
-      <c r="F29" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+      <c r="F29" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G29" s="0"/>
+      <c r="H29" s="0"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="s">
         <v>330</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="0" t="s">
         <v>56</v>
       </c>
-      <c r="C30">
+      <c r="C30" s="0">
         <v>0.38512075680995078</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D30" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="E30" t="s">
+      <c r="E30" s="0" t="s">
         <v>362</v>
       </c>
-      <c r="F30" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+      <c r="F30" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G30" s="0"/>
+      <c r="H30" s="0"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="s">
         <v>331</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="0" t="s">
         <v>56</v>
       </c>
-      <c r="C31">
-        <v>7.5217966021746033E-2</v>
-      </c>
-      <c r="D31" t="s">
+      <c r="C31" s="0">
+        <v>0.075217966021746033</v>
+      </c>
+      <c r="D31" s="0" t="s">
         <v>66</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E31" s="0" t="s">
         <v>363</v>
       </c>
-      <c r="F31" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+      <c r="F31" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G31" s="0"/>
+      <c r="H31" s="0"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="s">
         <v>332</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="0" t="s">
         <v>56</v>
       </c>
-      <c r="C32">
-        <v>7.5217966021746033E-2</v>
-      </c>
-      <c r="D32" t="s">
+      <c r="C32" s="0">
+        <v>0.075217966021746033</v>
+      </c>
+      <c r="D32" s="0" t="s">
         <v>66</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E32" s="0" t="s">
         <v>364</v>
       </c>
-      <c r="F32" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+      <c r="F32" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G32" s="0"/>
+      <c r="H32" s="0"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="s">
         <v>333</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="0" t="s">
         <v>56</v>
       </c>
-      <c r="C33">
+      <c r="C33" s="0">
         <v>0.28369565319769752</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D33" s="0" t="s">
         <v>59</v>
       </c>
-      <c r="E33" t="s">
+      <c r="E33" s="0" t="s">
         <v>365</v>
       </c>
-      <c r="F33" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+      <c r="F33" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G33" s="0"/>
+      <c r="H33" s="0"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="s">
         <v>334</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B34" s="0" t="s">
         <v>56</v>
       </c>
-      <c r="C34">
+      <c r="C34" s="0">
         <v>0.26513612448382945</v>
       </c>
-      <c r="D34" t="s">
+      <c r="D34" s="0" t="s">
         <v>59</v>
       </c>
-      <c r="E34" t="s">
+      <c r="E34" s="0" t="s">
         <v>366</v>
       </c>
-      <c r="F34" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+      <c r="F34" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G34" s="0"/>
+      <c r="H34" s="0"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="s">
         <v>388</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B35" s="0" t="s">
         <v>56</v>
       </c>
-      <c r="C35">
-        <v>2.8568191064456228E-2</v>
-      </c>
-      <c r="F35" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+      <c r="C35" s="0">
+        <v>0.028568191064456228</v>
+      </c>
+      <c r="D35" s="0"/>
+      <c r="E35" s="0"/>
+      <c r="F35" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G35" s="0"/>
+      <c r="H35" s="0"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="s">
         <v>389</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B36" s="0" t="s">
         <v>56</v>
       </c>
-      <c r="C36">
+      <c r="C36" s="0">
         <v>0.23237691205670161</v>
       </c>
-      <c r="F36" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+      <c r="D36" s="0"/>
+      <c r="E36" s="0"/>
+      <c r="F36" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G36" s="0"/>
+      <c r="H36" s="0"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="s">
         <v>390</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B37" s="0" t="s">
         <v>56</v>
       </c>
-      <c r="C37">
+      <c r="C37" s="0">
         <v>0.3614852233974003</v>
       </c>
-      <c r="F37" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+      <c r="D37" s="0"/>
+      <c r="E37" s="0"/>
+      <c r="F37" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G37" s="0"/>
+      <c r="H37" s="0"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="s">
         <v>391</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B38" s="0" t="s">
         <v>56</v>
       </c>
-      <c r="C38">
+      <c r="C38" s="0">
         <v>0.21148522339740031</v>
       </c>
-      <c r="F38" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+      <c r="D38" s="0"/>
+      <c r="E38" s="0"/>
+      <c r="F38" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G38" s="0"/>
+      <c r="H38" s="0"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="s">
         <v>165</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="C39">
+      <c r="C39" s="0">
         <v>4.8546281926201837</v>
       </c>
-      <c r="F39" t="s">
+      <c r="D39" s="0"/>
+      <c r="E39" s="0"/>
+      <c r="F39" s="0" t="s">
         <v>376</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+      <c r="G39" s="0"/>
+      <c r="H39" s="0"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="s">
         <v>335</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B40" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="C40">
+      <c r="C40" s="0">
         <v>22.737783592977756</v>
       </c>
-      <c r="D40" t="s">
+      <c r="D40" s="0" t="s">
         <v>135</v>
       </c>
-      <c r="E40" t="s">
+      <c r="E40" s="0" t="s">
         <v>367</v>
       </c>
-      <c r="F40" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+      <c r="F40" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G40" s="0"/>
+      <c r="H40" s="0"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="s">
         <v>336</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B41" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="C41">
+      <c r="C41" s="0">
         <v>11</v>
       </c>
-      <c r="D41" t="s">
+      <c r="D41" s="0" t="s">
         <v>135</v>
       </c>
-      <c r="E41" t="s">
+      <c r="E41" s="0" t="s">
         <v>368</v>
       </c>
-      <c r="F41" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+      <c r="F41" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G41" s="0"/>
+      <c r="H41" s="0"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="s">
         <v>337</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B42" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="C42">
+      <c r="C42" s="0">
         <v>14.810748414335091</v>
       </c>
-      <c r="D42" t="s">
+      <c r="D42" s="0" t="s">
         <v>135</v>
       </c>
-      <c r="E42" t="s">
+      <c r="E42" s="0" t="s">
         <v>369</v>
       </c>
-      <c r="F42" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
+      <c r="F42" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G42" s="0"/>
+      <c r="H42" s="0"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="s">
         <v>338</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B43" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="C43">
+      <c r="C43" s="0">
         <v>12.24744871391589</v>
       </c>
-      <c r="D43" t="s">
+      <c r="D43" s="0" t="s">
         <v>135</v>
       </c>
-      <c r="E43" t="s">
+      <c r="E43" s="0" t="s">
         <v>370</v>
       </c>
-      <c r="F43" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
+      <c r="F43" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G43" s="0"/>
+      <c r="H43" s="0"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="s">
         <v>339</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B44" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="C44">
+      <c r="C44" s="0">
         <v>48.189685104221404</v>
       </c>
-      <c r="D44" t="s">
+      <c r="D44" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="E44" t="s">
+      <c r="E44" s="0" t="s">
         <v>371</v>
       </c>
-      <c r="F44" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
+      <c r="F44" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G44" s="0"/>
+      <c r="H44" s="0"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="s">
         <v>340</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B45" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="C45">
+      <c r="C45" s="0">
         <v>16.699244233993625</v>
       </c>
-      <c r="D45" t="s">
+      <c r="D45" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="E45" t="s">
+      <c r="E45" s="0" t="s">
         <v>372</v>
       </c>
-      <c r="F45" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
+      <c r="F45" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G45" s="0"/>
+      <c r="H45" s="0"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="s">
         <v>341</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B46" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="C46">
+      <c r="C46" s="0">
         <v>47.623902569604006</v>
       </c>
-      <c r="D46" t="s">
+      <c r="D46" s="0" t="s">
         <v>345</v>
       </c>
-      <c r="E46" t="s">
+      <c r="E46" s="0" t="s">
         <v>373</v>
       </c>
-      <c r="F46" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
+      <c r="F46" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G46" s="0"/>
+      <c r="H46" s="0"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="s">
         <v>342</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B47" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="C47">
+      <c r="C47" s="0">
         <v>0.4509256385240365</v>
       </c>
-      <c r="F47" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
+      <c r="D47" s="0"/>
+      <c r="E47" s="0"/>
+      <c r="F47" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G47" s="0"/>
+      <c r="H47" s="0"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="s">
         <v>343</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B48" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="C48">
+      <c r="C48" s="0">
         <v>237637.81150216723</v>
       </c>
-      <c r="F48" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
+      <c r="D48" s="0"/>
+      <c r="E48" s="0"/>
+      <c r="F48" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G48" s="0"/>
+      <c r="H48" s="0"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="s">
         <v>344</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B49" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="C49">
+      <c r="C49" s="0">
         <v>133077.17444121366</v>
       </c>
-      <c r="F49" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
+      <c r="D49" s="0"/>
+      <c r="E49" s="0"/>
+      <c r="F49" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G49" s="0"/>
+      <c r="H49" s="0"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="s">
         <v>392</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B50" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="C50">
-        <v>34.655879425474303</v>
-      </c>
-      <c r="F50" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
+      <c r="C50" s="0">
+        <v>34.655879425474304</v>
+      </c>
+      <c r="D50" s="0"/>
+      <c r="E50" s="0"/>
+      <c r="F50" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G50" s="0"/>
+      <c r="H50" s="0"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="s">
         <v>393</v>
       </c>
-      <c r="B51" t="s">
+      <c r="B51" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="C51">
+      <c r="C51" s="0">
         <v>15.682651825415947</v>
       </c>
-      <c r="F51" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
+      <c r="D51" s="0"/>
+      <c r="E51" s="0"/>
+      <c r="F51" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G51" s="0"/>
+      <c r="H51" s="0"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="0" t="s">
         <v>394</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B52" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="C52">
-        <v>3.8</v>
-      </c>
-      <c r="F52" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
+      <c r="C52" s="0">
+        <v>3.7999999999999998</v>
+      </c>
+      <c r="D52" s="0"/>
+      <c r="E52" s="0"/>
+      <c r="F52" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G52" s="0"/>
+      <c r="H52" s="0"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="0" t="s">
         <v>395</v>
       </c>
-      <c r="B53" t="s">
+      <c r="B53" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="C53">
+      <c r="C53" s="0">
         <v>-1.52</v>
       </c>
-      <c r="F53" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
+      <c r="D53" s="0"/>
+      <c r="E53" s="0"/>
+      <c r="F53" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G53" s="0"/>
+      <c r="H53" s="0"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="0" t="s">
         <v>396</v>
       </c>
-      <c r="B54" t="s">
+      <c r="B54" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="C54">
+      <c r="C54" s="0">
         <v>5.6999999999999993</v>
       </c>
-      <c r="F54" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
+      <c r="D54" s="0"/>
+      <c r="E54" s="0"/>
+      <c r="F54" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G54" s="0"/>
+      <c r="H54" s="0"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="0" t="s">
         <v>397</v>
       </c>
-      <c r="B55" t="s">
+      <c r="B55" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="C55">
-        <v>-2.2800000000000002</v>
-      </c>
-      <c r="F55" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
+      <c r="C55" s="0">
+        <v>-2.2800000000000003</v>
+      </c>
+      <c r="D55" s="0"/>
+      <c r="E55" s="0"/>
+      <c r="F55" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G55" s="0"/>
+      <c r="H55" s="0"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="0" t="s">
         <v>398</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B56" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="C56">
+      <c r="C56" s="0">
         <v>16.966129707239677</v>
       </c>
-      <c r="F56" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
+      <c r="D56" s="0"/>
+      <c r="E56" s="0"/>
+      <c r="F56" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G56" s="0"/>
+      <c r="H56" s="0"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="0" t="s">
         <v>399</v>
       </c>
-      <c r="B57" t="s">
+      <c r="B57" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="C57">
+      <c r="C57" s="0">
         <v>24.931681951672573</v>
       </c>
-      <c r="F57" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
+      <c r="D57" s="0"/>
+      <c r="E57" s="0"/>
+      <c r="F57" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G57" s="0"/>
+      <c r="H57" s="0"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="0" t="s">
         <v>400</v>
       </c>
-      <c r="B58" t="s">
+      <c r="B58" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="C58">
+      <c r="C58" s="0">
         <v>38.987864353658594</v>
       </c>
-      <c r="F58" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
+      <c r="D58" s="0"/>
+      <c r="E58" s="0"/>
+      <c r="F58" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G58" s="0"/>
+      <c r="H58" s="0"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="0" t="s">
         <v>401</v>
       </c>
-      <c r="B59" t="s">
+      <c r="B59" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="C59">
+      <c r="C59" s="0">
         <v>43.319849281842878</v>
       </c>
-      <c r="F59" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
+      <c r="D59" s="0"/>
+      <c r="E59" s="0"/>
+      <c r="F59" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G59" s="0"/>
+      <c r="H59" s="0"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="0" t="s">
         <v>402</v>
       </c>
-      <c r="B60" t="s">
+      <c r="B60" s="0" t="s">
         <v>134</v>
       </c>
-      <c r="C60">
+      <c r="C60" s="0">
         <v>3.6377414361906815</v>
       </c>
-      <c r="F60" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
+      <c r="D60" s="0"/>
+      <c r="E60" s="0"/>
+      <c r="F60" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G60" s="0"/>
+      <c r="H60" s="0"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="0" t="s">
         <v>403</v>
       </c>
-      <c r="B61" t="s">
+      <c r="B61" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C61">
-        <v>27.630496754505511</v>
-      </c>
-      <c r="F61" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
+      <c r="C61" s="0">
+        <v>27.630496754505508</v>
+      </c>
+      <c r="D61" s="0"/>
+      <c r="E61" s="0"/>
+      <c r="F61" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G61" s="0"/>
+      <c r="H61" s="0"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="0" t="s">
         <v>404</v>
       </c>
-      <c r="B62" t="s">
+      <c r="B62" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C62">
+      <c r="C62" s="0">
         <v>0</v>
       </c>
-      <c r="F62" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
+      <c r="D62" s="0"/>
+      <c r="E62" s="0"/>
+      <c r="F62" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G62" s="0"/>
+      <c r="H62" s="0"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="0" t="s">
         <v>405</v>
       </c>
-      <c r="B63" t="s">
+      <c r="B63" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C63" t="s">
+      <c r="C63" s="0" t="s">
         <v>451</v>
       </c>
-      <c r="F63" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
+      <c r="D63" s="0"/>
+      <c r="E63" s="0"/>
+      <c r="F63" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G63" s="0"/>
+      <c r="H63" s="0"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="0" t="s">
         <v>406</v>
       </c>
-      <c r="B64" t="s">
+      <c r="B64" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C64">
+      <c r="C64" s="0">
         <v>72.102440957348392</v>
       </c>
-      <c r="F64" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
+      <c r="D64" s="0"/>
+      <c r="E64" s="0"/>
+      <c r="F64" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G64" s="0"/>
+      <c r="H64" s="0"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="0" t="s">
         <v>407</v>
       </c>
-      <c r="B65" t="s">
+      <c r="B65" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C65">
+      <c r="C65" s="0">
         <v>0</v>
       </c>
-      <c r="F65" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
+      <c r="D65" s="0"/>
+      <c r="E65" s="0"/>
+      <c r="F65" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G65" s="0"/>
+      <c r="H65" s="0"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="0" t="s">
         <v>408</v>
       </c>
-      <c r="B66" t="s">
+      <c r="B66" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C66">
-        <v>-1.319188550096897</v>
-      </c>
-      <c r="F66" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
+      <c r="C66" s="0">
+        <v>-1.3191885500968961</v>
+      </c>
+      <c r="D66" s="0"/>
+      <c r="E66" s="0"/>
+      <c r="F66" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G66" s="0"/>
+      <c r="H66" s="0"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="0" t="s">
         <v>409</v>
       </c>
-      <c r="B67" t="s">
+      <c r="B67" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C67">
+      <c r="C67" s="0">
         <v>0</v>
       </c>
-      <c r="F67" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
+      <c r="D67" s="0"/>
+      <c r="E67" s="0"/>
+      <c r="F67" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G67" s="0"/>
+      <c r="H67" s="0"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="0" t="s">
         <v>410</v>
       </c>
-      <c r="B68" t="s">
+      <c r="B68" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C68">
-        <v>4.2603031906991697</v>
-      </c>
-      <c r="F68" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
+      <c r="C68" s="0">
+        <v>4.2603031906991689</v>
+      </c>
+      <c r="D68" s="0"/>
+      <c r="E68" s="0"/>
+      <c r="F68" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G68" s="0"/>
+      <c r="H68" s="0"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="0" t="s">
         <v>411</v>
       </c>
-      <c r="B69" t="s">
+      <c r="B69" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C69">
+      <c r="C69" s="0">
         <v>0</v>
       </c>
-      <c r="F69" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
+      <c r="D69" s="0"/>
+      <c r="E69" s="0"/>
+      <c r="F69" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G69" s="0"/>
+      <c r="H69" s="0"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="0" t="s">
         <v>412</v>
       </c>
-      <c r="B70" t="s">
+      <c r="B70" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C70">
+      <c r="C70" s="0">
         <v>5.6725107333819</v>
       </c>
-      <c r="F70" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
+      <c r="D70" s="0"/>
+      <c r="E70" s="0"/>
+      <c r="F70" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G70" s="0"/>
+      <c r="H70" s="0"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="0" t="s">
         <v>413</v>
       </c>
-      <c r="B71" t="s">
+      <c r="B71" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C71">
+      <c r="C71" s="0">
         <v>5.9726584296289333</v>
       </c>
-      <c r="F71" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
+      <c r="D71" s="0"/>
+      <c r="E71" s="0"/>
+      <c r="F71" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G71" s="0"/>
+      <c r="H71" s="0"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="0" t="s">
         <v>414</v>
       </c>
-      <c r="B72" t="s">
+      <c r="B72" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C72">
+      <c r="C72" s="0">
         <v>26.62280764138869</v>
       </c>
-      <c r="F72" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
+      <c r="D72" s="0"/>
+      <c r="E72" s="0"/>
+      <c r="F72" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G72" s="0"/>
+      <c r="H72" s="0"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="0" t="s">
         <v>482</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B73" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C73">
+      <c r="C73" s="0">
         <v>47.120013524581758</v>
       </c>
-      <c r="F73" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
+      <c r="D73" s="0"/>
+      <c r="E73" s="0"/>
+      <c r="F73" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G73" s="0"/>
+      <c r="H73" s="0"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="0" t="s">
         <v>415</v>
       </c>
-      <c r="B74" t="s">
+      <c r="B74" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C74">
+      <c r="C74" s="0">
         <v>15.78851883984732</v>
       </c>
-      <c r="F74" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
+      <c r="D74" s="0"/>
+      <c r="E74" s="0"/>
+      <c r="F74" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G74" s="0"/>
+      <c r="H74" s="0"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="0" t="s">
         <v>416</v>
       </c>
-      <c r="B75" t="s">
+      <c r="B75" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C75">
+      <c r="C75" s="0">
         <v>0.38346429214607308</v>
       </c>
-      <c r="F75" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
+      <c r="D75" s="0"/>
+      <c r="E75" s="0"/>
+      <c r="F75" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G75" s="0"/>
+      <c r="H75" s="0"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="0" t="s">
         <v>417</v>
       </c>
-      <c r="B76" t="s">
+      <c r="B76" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C76" t="s">
+      <c r="C76" s="0" t="s">
         <v>490</v>
       </c>
-      <c r="F76" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
+      <c r="D76" s="0"/>
+      <c r="E76" s="0"/>
+      <c r="F76" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G76" s="0"/>
+      <c r="H76" s="0"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="0" t="s">
         <v>418</v>
       </c>
-      <c r="B77" t="s">
+      <c r="B77" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C77">
+      <c r="C77" s="0">
         <v>210.59818457285559</v>
       </c>
-      <c r="F77" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
+      <c r="D77" s="0"/>
+      <c r="E77" s="0"/>
+      <c r="F77" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G77" s="0"/>
+      <c r="H77" s="0"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="0" t="s">
         <v>419</v>
       </c>
-      <c r="B78" t="s">
+      <c r="B78" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C78">
+      <c r="C78" s="0">
         <v>0.249319539769885</v>
       </c>
-      <c r="F78" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
+      <c r="D78" s="0"/>
+      <c r="E78" s="0"/>
+      <c r="F78" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G78" s="0"/>
+      <c r="H78" s="0"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="0" t="s">
         <v>420</v>
       </c>
-      <c r="B79" t="s">
+      <c r="B79" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C79" t="s">
+      <c r="C79" s="0" t="s">
         <v>452</v>
       </c>
-      <c r="F79" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
+      <c r="D79" s="0"/>
+      <c r="E79" s="0"/>
+      <c r="F79" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G79" s="0"/>
+      <c r="H79" s="0"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="0" t="s">
         <v>421</v>
       </c>
-      <c r="B80" t="s">
+      <c r="B80" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C80">
+      <c r="C80" s="0">
         <v>10.35552938735983</v>
       </c>
-      <c r="F80" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
+      <c r="D80" s="0"/>
+      <c r="E80" s="0"/>
+      <c r="F80" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G80" s="0"/>
+      <c r="H80" s="0"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="0" t="s">
         <v>422</v>
       </c>
-      <c r="B81" t="s">
+      <c r="B81" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C81">
+      <c r="C81" s="0">
         <v>323.73645427492852</v>
       </c>
-      <c r="F81" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
+      <c r="D81" s="0"/>
+      <c r="E81" s="0"/>
+      <c r="F81" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G81" s="0"/>
+      <c r="H81" s="0"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="0" t="s">
         <v>423</v>
       </c>
-      <c r="B82" t="s">
+      <c r="B82" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C82">
+      <c r="C82" s="0">
         <v>20.793297705941828</v>
       </c>
-      <c r="F82" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
+      <c r="D82" s="0"/>
+      <c r="E82" s="0"/>
+      <c r="F82" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G82" s="0"/>
+      <c r="H82" s="0"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="0" t="s">
         <v>424</v>
       </c>
-      <c r="B83" t="s">
+      <c r="B83" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C83">
+      <c r="C83" s="0">
         <v>0.30965445458432234</v>
       </c>
-      <c r="F83" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
+      <c r="D83" s="0"/>
+      <c r="E83" s="0"/>
+      <c r="F83" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G83" s="0"/>
+      <c r="H83" s="0"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="0" t="s">
         <v>425</v>
       </c>
-      <c r="B84" t="s">
+      <c r="B84" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C84">
+      <c r="C84" s="0">
         <v>3.3914500000000003</v>
       </c>
-      <c r="F84" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
+      <c r="D84" s="0"/>
+      <c r="E84" s="0"/>
+      <c r="F84" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G84" s="0"/>
+      <c r="H84" s="0"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="0" t="s">
         <v>426</v>
       </c>
-      <c r="B85" t="s">
+      <c r="B85" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C85">
+      <c r="C85" s="0">
         <v>33.270124500000001</v>
       </c>
-      <c r="F85" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
+      <c r="D85" s="0"/>
+      <c r="E85" s="0"/>
+      <c r="F85" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G85" s="0"/>
+      <c r="H85" s="0"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="0" t="s">
         <v>427</v>
       </c>
-      <c r="B86" t="s">
+      <c r="B86" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C86">
+      <c r="C86" s="0">
         <v>16.616876525517039</v>
       </c>
-      <c r="F86" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
+      <c r="D86" s="0"/>
+      <c r="E86" s="0"/>
+      <c r="F86" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G86" s="0"/>
+      <c r="H86" s="0"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="0" t="s">
         <v>428</v>
       </c>
-      <c r="B87" t="s">
+      <c r="B87" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C87">
-        <v>7.8800000000000009E-2</v>
-      </c>
-      <c r="F87" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
+      <c r="C87" s="0">
+        <v>0.078800000000000009</v>
+      </c>
+      <c r="D87" s="0"/>
+      <c r="E87" s="0"/>
+      <c r="F87" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G87" s="0"/>
+      <c r="H87" s="0"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="0" t="s">
         <v>429</v>
       </c>
-      <c r="B88" t="s">
+      <c r="B88" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C88">
-        <v>51.753621214228787</v>
-      </c>
-      <c r="F88" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
+      <c r="C88" s="0">
+        <v>51.753621214228794</v>
+      </c>
+      <c r="D88" s="0"/>
+      <c r="E88" s="0"/>
+      <c r="F88" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G88" s="0"/>
+      <c r="H88" s="0"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="0" t="s">
         <v>492</v>
       </c>
-      <c r="B89" t="s">
+      <c r="B89" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C89">
-        <v>182.17938531024632</v>
-      </c>
-      <c r="F89" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
+      <c r="C89" s="0">
+        <v>182.17938531024629</v>
+      </c>
+      <c r="D89" s="0"/>
+      <c r="E89" s="0"/>
+      <c r="F89" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G89" s="0"/>
+      <c r="H89" s="0"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="0" t="s">
         <v>493</v>
       </c>
-      <c r="B90" t="s">
+      <c r="B90" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C90">
+      <c r="C90" s="0">
         <v>3.5283725544652502</v>
       </c>
-      <c r="F90" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
+      <c r="D90" s="0"/>
+      <c r="E90" s="0"/>
+      <c r="F90" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G90" s="0"/>
+      <c r="H90" s="0"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="0" t="s">
         <v>494</v>
       </c>
-      <c r="B91" t="s">
+      <c r="B91" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C91">
-        <v>5.1976901145282772</v>
-      </c>
-      <c r="F91" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
+      <c r="C91" s="0">
+        <v>5.1976901145282737</v>
+      </c>
+      <c r="D91" s="0"/>
+      <c r="E91" s="0"/>
+      <c r="F91" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G91" s="0"/>
+      <c r="H91" s="0"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="0" t="s">
         <v>495</v>
       </c>
-      <c r="B92" t="s">
+      <c r="B92" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C92">
-        <v>182.4016896292334</v>
-      </c>
-      <c r="F92" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
+      <c r="C92" s="0">
+        <v>182.40168962923338</v>
+      </c>
+      <c r="D92" s="0"/>
+      <c r="E92" s="0"/>
+      <c r="F92" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G92" s="0"/>
+      <c r="H92" s="0"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="0" t="s">
         <v>496</v>
       </c>
-      <c r="B93" t="s">
+      <c r="B93" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C93">
-        <v>8.7260626689935279</v>
-      </c>
-      <c r="F93" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
+      <c r="C93" s="0">
+        <v>8.7260626689935226</v>
+      </c>
+      <c r="D93" s="0"/>
+      <c r="E93" s="0"/>
+      <c r="F93" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G93" s="0"/>
+      <c r="H93" s="0"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="0" t="s">
         <v>483</v>
       </c>
-      <c r="B94" t="s">
+      <c r="B94" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C94">
-        <v>0.32125969057566839</v>
-      </c>
-      <c r="F94" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
+      <c r="C94" s="0">
+        <v>0.32125969057566861</v>
+      </c>
+      <c r="D94" s="0"/>
+      <c r="E94" s="0"/>
+      <c r="F94" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G94" s="0"/>
+      <c r="H94" s="0"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="0" t="s">
         <v>484</v>
       </c>
-      <c r="B95" t="s">
+      <c r="B95" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C95">
-        <v>20.315455441423438</v>
-      </c>
-      <c r="F95" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
+      <c r="C95" s="0">
+        <v>20.315455441423445</v>
+      </c>
+      <c r="D95" s="0"/>
+      <c r="E95" s="0"/>
+      <c r="F95" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G95" s="0"/>
+      <c r="H95" s="0"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="0" t="s">
         <v>519</v>
       </c>
-      <c r="B96" t="s">
+      <c r="B96" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C96">
+      <c r="C96" s="0">
         <v>4.3293357933508361</v>
       </c>
-      <c r="F96" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
+      <c r="D96" s="0"/>
+      <c r="E96" s="0"/>
+      <c r="F96" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G96" s="0"/>
+      <c r="H96" s="0"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="0" t="s">
         <v>520</v>
       </c>
-      <c r="B97" t="s">
+      <c r="B97" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C97">
-        <v>2.846137178026887E-2</v>
-      </c>
-      <c r="F97" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
+      <c r="C97" s="0">
+        <v>0.02846137178026887</v>
+      </c>
+      <c r="D97" s="0"/>
+      <c r="E97" s="0"/>
+      <c r="F97" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G97" s="0"/>
+      <c r="H97" s="0"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="0" t="s">
         <v>497</v>
       </c>
-      <c r="B98" t="s">
+      <c r="B98" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C98">
+      <c r="C98" s="0">
         <v>175.53527084344745</v>
       </c>
-      <c r="F98" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
+      <c r="D98" s="0"/>
+      <c r="E98" s="0"/>
+      <c r="F98" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G98" s="0"/>
+      <c r="H98" s="0"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="0" t="s">
         <v>498</v>
       </c>
-      <c r="B99" t="s">
+      <c r="B99" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C99">
+      <c r="C99" s="0">
         <v>2.3058437450753382</v>
       </c>
-      <c r="F99" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
+      <c r="D99" s="0"/>
+      <c r="E99" s="0"/>
+      <c r="F99" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G99" s="0"/>
+      <c r="H99" s="0"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="0" t="s">
         <v>499</v>
       </c>
-      <c r="B100" t="s">
+      <c r="B100" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C100">
+      <c r="C100" s="0">
         <v>23.532669135777482</v>
       </c>
-      <c r="F100" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
+      <c r="D100" s="0"/>
+      <c r="E100" s="0"/>
+      <c r="F100" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G100" s="0"/>
+      <c r="H100" s="0"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="0" t="s">
         <v>500</v>
       </c>
-      <c r="B101" t="s">
+      <c r="B101" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C101">
-        <v>180.20541295988968</v>
-      </c>
-      <c r="F101" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A102" t="s">
+      <c r="C101" s="0">
+        <v>180.20541295988969</v>
+      </c>
+      <c r="D101" s="0"/>
+      <c r="E101" s="0"/>
+      <c r="F101" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G101" s="0"/>
+      <c r="H101" s="0"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="0" t="s">
         <v>501</v>
       </c>
-      <c r="B102" t="s">
+      <c r="B102" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C102">
+      <c r="C102" s="0">
         <v>25.838512880852818</v>
       </c>
-      <c r="F102" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A103" t="s">
+      <c r="D102" s="0"/>
+      <c r="E102" s="0"/>
+      <c r="F102" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G102" s="0"/>
+      <c r="H102" s="0"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="0" t="s">
         <v>485</v>
       </c>
-      <c r="B103" t="s">
+      <c r="B103" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C103">
+      <c r="C103" s="0">
         <v>0.33736271314803434</v>
       </c>
-      <c r="F103" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A104" t="s">
+      <c r="D103" s="0"/>
+      <c r="E103" s="0"/>
+      <c r="F103" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G103" s="0"/>
+      <c r="H103" s="0"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="0" t="s">
         <v>486</v>
       </c>
-      <c r="B104" t="s">
+      <c r="B104" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C104">
+      <c r="C104" s="0">
         <v>6.1985566993614434</v>
       </c>
-      <c r="F104" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A105" t="s">
+      <c r="D104" s="0"/>
+      <c r="E104" s="0"/>
+      <c r="F104" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G104" s="0"/>
+      <c r="H104" s="0"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="0" t="s">
         <v>502</v>
       </c>
-      <c r="B105" t="s">
+      <c r="B105" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C105">
+      <c r="C105" s="0">
         <v>0.46957187967523628</v>
       </c>
-      <c r="F105" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A106" t="s">
+      <c r="D105" s="0"/>
+      <c r="E105" s="0"/>
+      <c r="F105" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G105" s="0"/>
+      <c r="H105" s="0"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="0" t="s">
         <v>503</v>
       </c>
-      <c r="B106" t="s">
+      <c r="B106" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C106">
+      <c r="C106" s="0">
         <v>0.33682338763133246</v>
       </c>
-      <c r="F106" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A107" t="s">
+      <c r="D106" s="0"/>
+      <c r="E106" s="0"/>
+      <c r="F106" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G106" s="0"/>
+      <c r="H106" s="0"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="0" t="s">
         <v>504</v>
       </c>
-      <c r="B107" t="s">
+      <c r="B107" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C107">
+      <c r="C107" s="0">
         <v>0.11450290898458269</v>
       </c>
-      <c r="F107" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A108" t="s">
+      <c r="D107" s="0"/>
+      <c r="E107" s="0"/>
+      <c r="F107" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G107" s="0"/>
+      <c r="H107" s="0"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="0" t="s">
         <v>505</v>
       </c>
-      <c r="B108" t="s">
+      <c r="B108" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C108">
+      <c r="C108" s="0">
         <v>0.45132629661591511</v>
       </c>
-      <c r="F108" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A109" t="s">
+      <c r="D108" s="0"/>
+      <c r="E108" s="0"/>
+      <c r="F108" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G108" s="0"/>
+      <c r="H108" s="0"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="0" t="s">
         <v>487</v>
       </c>
-      <c r="B109" t="s">
+      <c r="B109" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C109">
+      <c r="C109" s="0">
         <v>62.887982433591418</v>
       </c>
-      <c r="F109" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A110" t="s">
+      <c r="D109" s="0"/>
+      <c r="E109" s="0"/>
+      <c r="F109" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G109" s="0"/>
+      <c r="H109" s="0"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="0" t="s">
         <v>488</v>
       </c>
-      <c r="B110" t="s">
+      <c r="B110" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C110">
+      <c r="C110" s="0">
         <v>20.049072635988303</v>
       </c>
-      <c r="F110" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A111" t="s">
+      <c r="D110" s="0"/>
+      <c r="E110" s="0"/>
+      <c r="F110" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G110" s="0"/>
+      <c r="H110" s="0"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="0" t="s">
         <v>506</v>
       </c>
-      <c r="B111" t="s">
+      <c r="B111" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C111">
+      <c r="C111" s="0">
         <v>216.54759148975538</v>
       </c>
-      <c r="F111" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A112" t="s">
+      <c r="D111" s="0"/>
+      <c r="E111" s="0"/>
+      <c r="F111" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G111" s="0"/>
+      <c r="H111" s="0"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="0" t="s">
         <v>507</v>
       </c>
-      <c r="B112" t="s">
+      <c r="B112" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C112">
+      <c r="C112" s="0">
         <v>2.0217106942854626</v>
       </c>
-      <c r="F112" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A113" t="s">
+      <c r="D112" s="0"/>
+      <c r="E112" s="0"/>
+      <c r="F112" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G112" s="0"/>
+      <c r="H112" s="0"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="0" t="s">
         <v>508</v>
       </c>
-      <c r="B113" t="s">
+      <c r="B113" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C113">
+      <c r="C113" s="0">
         <v>2.5446250468831417</v>
       </c>
-      <c r="F113" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A114" t="s">
+      <c r="D113" s="0"/>
+      <c r="E113" s="0"/>
+      <c r="F113" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G113" s="0"/>
+      <c r="H113" s="0"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="0" t="s">
         <v>514</v>
       </c>
-      <c r="B114" t="s">
+      <c r="B114" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C114">
+      <c r="C114" s="0">
         <v>0.10262510605021724</v>
       </c>
-      <c r="F114" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A115" t="s">
+      <c r="D114" s="0"/>
+      <c r="E114" s="0"/>
+      <c r="F114" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G114" s="0"/>
+      <c r="H114" s="0"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="0" t="s">
         <v>489</v>
       </c>
-      <c r="B115" t="s">
+      <c r="B115" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C115">
-        <v>72.095248444491872</v>
-      </c>
-      <c r="F115" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A116" t="s">
+      <c r="C115" s="0">
+        <v>72.095248444491873</v>
+      </c>
+      <c r="D115" s="0"/>
+      <c r="E115" s="0"/>
+      <c r="F115" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G115" s="0"/>
+      <c r="H115" s="0"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="0" t="s">
         <v>515</v>
       </c>
-      <c r="B116" t="s">
+      <c r="B116" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C116">
+      <c r="C116" s="0">
         <v>46.311829358431872</v>
       </c>
-      <c r="F116" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A117" t="s">
+      <c r="D116" s="0"/>
+      <c r="E116" s="0"/>
+      <c r="F116" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G116" s="0"/>
+      <c r="H116" s="0"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="0" t="s">
         <v>516</v>
       </c>
-      <c r="B117" t="s">
+      <c r="B117" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C117">
+      <c r="C117" s="0">
         <v>2.8019142042285794</v>
       </c>
-      <c r="F117" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A118" t="s">
+      <c r="D117" s="0"/>
+      <c r="E117" s="0"/>
+      <c r="F117" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G117" s="0"/>
+      <c r="H117" s="0"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="0" t="s">
         <v>523</v>
       </c>
-      <c r="B118" t="s">
+      <c r="B118" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C118">
+      <c r="C118" s="0">
         <v>0.19299193437653406</v>
       </c>
-      <c r="F118" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A119" t="s">
+      <c r="D118" s="0"/>
+      <c r="E118" s="0"/>
+      <c r="F118" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G118" s="0"/>
+      <c r="H118" s="0"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="0" t="s">
         <v>517</v>
       </c>
-      <c r="B119" t="s">
+      <c r="B119" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C119">
+      <c r="C119" s="0">
         <v>221.3736775163259</v>
       </c>
-      <c r="F119" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A120" t="s">
+      <c r="D119" s="0"/>
+      <c r="E119" s="0"/>
+      <c r="F119" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G119" s="0"/>
+      <c r="H119" s="0"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="0" t="s">
         <v>518</v>
       </c>
-      <c r="B120" t="s">
+      <c r="B120" s="0" t="s">
         <v>263</v>
       </c>
-      <c r="C120">
+      <c r="C120" s="0">
         <v>0.92725557606200626</v>
       </c>
-      <c r="F120" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A121" t="s">
+      <c r="D120" s="0"/>
+      <c r="E120" s="0"/>
+      <c r="F120" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G120" s="0"/>
+      <c r="H120" s="0"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="0" t="s">
         <v>430</v>
       </c>
-      <c r="B121" t="s">
+      <c r="B121" s="0" t="s">
         <v>450</v>
       </c>
-      <c r="C121">
-        <v>0.3</v>
-      </c>
-      <c r="F121" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A122" t="s">
+      <c r="C121" s="0">
+        <v>0.29999999999999999</v>
+      </c>
+      <c r="D121" s="0"/>
+      <c r="E121" s="0"/>
+      <c r="F121" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G121" s="0"/>
+      <c r="H121" s="0"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="0" t="s">
         <v>431</v>
       </c>
-      <c r="B122" t="s">
+      <c r="B122" s="0" t="s">
         <v>450</v>
       </c>
-      <c r="C122">
+      <c r="C122" s="0">
         <v>27.176996615837602</v>
       </c>
-      <c r="F122" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A123" t="s">
+      <c r="D122" s="0"/>
+      <c r="E122" s="0"/>
+      <c r="F122" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G122" s="0"/>
+      <c r="H122" s="0"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="0" t="s">
         <v>432</v>
       </c>
-      <c r="B123" t="s">
+      <c r="B123" s="0" t="s">
         <v>450</v>
       </c>
-      <c r="C123">
+      <c r="C123" s="0">
         <v>2.8230033841623978</v>
       </c>
-      <c r="F123" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A124" t="s">
+      <c r="D123" s="0"/>
+      <c r="E123" s="0"/>
+      <c r="F123" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G123" s="0"/>
+      <c r="H123" s="0"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="0" t="s">
         <v>433</v>
       </c>
-      <c r="B124" t="s">
+      <c r="B124" s="0" t="s">
         <v>450</v>
       </c>
-      <c r="C124">
+      <c r="C124" s="0">
         <v>0.25</v>
       </c>
-      <c r="F124" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A125" t="s">
+      <c r="D124" s="0"/>
+      <c r="E124" s="0"/>
+      <c r="F124" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G124" s="0"/>
+      <c r="H124" s="0"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="0" t="s">
         <v>434</v>
       </c>
-      <c r="B125" t="s">
+      <c r="B125" s="0" t="s">
         <v>450</v>
       </c>
-      <c r="C125">
-        <v>0.7</v>
-      </c>
-      <c r="F125" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A126" t="s">
+      <c r="C125" s="0">
+        <v>0.69999999999999996</v>
+      </c>
+      <c r="D125" s="0"/>
+      <c r="E125" s="0"/>
+      <c r="F125" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G125" s="0"/>
+      <c r="H125" s="0"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="0" t="s">
         <v>435</v>
       </c>
-      <c r="B126" t="s">
+      <c r="B126" s="0" t="s">
         <v>450</v>
       </c>
-      <c r="C126">
+      <c r="C126" s="0">
         <v>1</v>
       </c>
-      <c r="F126" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A127" t="s">
+      <c r="D126" s="0"/>
+      <c r="E126" s="0"/>
+      <c r="F126" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G126" s="0"/>
+      <c r="H126" s="0"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="0" t="s">
         <v>436</v>
       </c>
-      <c r="B127" t="s">
+      <c r="B127" s="0" t="s">
         <v>450</v>
       </c>
-      <c r="C127">
+      <c r="C127" s="0">
         <v>0.12043337304073547</v>
       </c>
-      <c r="F127" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A128" t="s">
+      <c r="D127" s="0"/>
+      <c r="E127" s="0"/>
+      <c r="F127" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G127" s="0"/>
+      <c r="H127" s="0"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="0" t="s">
         <v>437</v>
       </c>
-      <c r="B128" t="s">
+      <c r="B128" s="0" t="s">
         <v>450</v>
       </c>
-      <c r="C128">
+      <c r="C128" s="0">
         <v>119.60561578781872</v>
       </c>
-      <c r="F128" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A129" t="s">
+      <c r="D128" s="0"/>
+      <c r="E128" s="0"/>
+      <c r="F128" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G128" s="0"/>
+      <c r="H128" s="0"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="0" t="s">
         <v>438</v>
       </c>
-      <c r="B129" t="s">
+      <c r="B129" s="0" t="s">
         <v>450</v>
       </c>
-      <c r="C129">
-        <v>7.5217966021746033E-2</v>
-      </c>
-      <c r="F129" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A130" t="s">
+      <c r="C129" s="0">
+        <v>0.075217966021746033</v>
+      </c>
+      <c r="D129" s="0"/>
+      <c r="E129" s="0"/>
+      <c r="F129" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G129" s="0"/>
+      <c r="H129" s="0"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="0" t="s">
         <v>439</v>
       </c>
-      <c r="B130" t="s">
+      <c r="B130" s="0" t="s">
         <v>450</v>
       </c>
-      <c r="C130">
-        <v>1.07</v>
-      </c>
-      <c r="F130" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A131" t="s">
+      <c r="C130" s="0">
+        <v>1.0700000000000001</v>
+      </c>
+      <c r="D130" s="0"/>
+      <c r="E130" s="0"/>
+      <c r="F130" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G130" s="0"/>
+      <c r="H130" s="0"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="0" t="s">
         <v>440</v>
       </c>
-      <c r="B131" t="s">
+      <c r="B131" s="0" t="s">
         <v>450</v>
       </c>
-      <c r="C131">
-        <v>0.3</v>
-      </c>
-      <c r="F131" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A132" t="s">
+      <c r="C131" s="0">
+        <v>0.29999999999999999</v>
+      </c>
+      <c r="D131" s="0"/>
+      <c r="E131" s="0"/>
+      <c r="F131" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G131" s="0"/>
+      <c r="H131" s="0"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="0" t="s">
         <v>441</v>
       </c>
-      <c r="B132" t="s">
+      <c r="B132" s="0" t="s">
         <v>450</v>
       </c>
-      <c r="C132">
+      <c r="C132" s="0">
         <v>29.162154556467332</v>
       </c>
-      <c r="F132" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A133" t="s">
+      <c r="D132" s="0"/>
+      <c r="E132" s="0"/>
+      <c r="F132" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G132" s="0"/>
+      <c r="H132" s="0"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="0" t="s">
         <v>442</v>
       </c>
-      <c r="B133" t="s">
+      <c r="B133" s="0" t="s">
         <v>450</v>
       </c>
-      <c r="C133">
+      <c r="C133" s="0">
         <v>0.83784544353266455</v>
       </c>
-      <c r="F133" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A134" t="s">
+      <c r="D133" s="0"/>
+      <c r="E133" s="0"/>
+      <c r="F133" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G133" s="0"/>
+      <c r="H133" s="0"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="0" t="s">
         <v>443</v>
       </c>
-      <c r="B134" t="s">
+      <c r="B134" s="0" t="s">
         <v>450</v>
       </c>
-      <c r="C134">
+      <c r="C134" s="0">
         <v>5.2033621722920103</v>
       </c>
-      <c r="F134" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A135" t="s">
+      <c r="D134" s="0"/>
+      <c r="E134" s="0"/>
+      <c r="F134" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G134" s="0"/>
+      <c r="H134" s="0"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="0" t="s">
         <v>444</v>
       </c>
-      <c r="B135" t="s">
+      <c r="B135" s="0" t="s">
         <v>450</v>
       </c>
-      <c r="C135">
+      <c r="C135" s="0">
         <v>0.3614852233974003</v>
       </c>
-      <c r="F135" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A136" t="s">
+      <c r="D135" s="0"/>
+      <c r="E135" s="0"/>
+      <c r="F135" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G135" s="0"/>
+      <c r="H135" s="0"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="0" t="s">
         <v>445</v>
       </c>
-      <c r="B136" t="s">
+      <c r="B136" s="0" t="s">
         <v>450</v>
       </c>
-      <c r="C136">
+      <c r="C136" s="0">
         <v>0.15</v>
       </c>
-      <c r="F136" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A137" t="s">
+      <c r="D136" s="0"/>
+      <c r="E136" s="0"/>
+      <c r="F136" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G136" s="0"/>
+      <c r="H136" s="0"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="0" t="s">
         <v>446</v>
       </c>
-      <c r="B137" t="s">
+      <c r="B137" s="0" t="s">
         <v>450</v>
       </c>
-      <c r="C137">
+      <c r="C137" s="0">
         <v>-0.78050432584380147</v>
       </c>
-      <c r="F137" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A138" t="s">
+      <c r="D137" s="0"/>
+      <c r="E137" s="0"/>
+      <c r="F137" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G137" s="0"/>
+      <c r="H137" s="0"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="0" t="s">
         <v>447</v>
       </c>
-      <c r="B138" t="s">
+      <c r="B138" s="0" t="s">
         <v>450</v>
       </c>
-      <c r="C138">
+      <c r="C138" s="0">
         <v>0.12602616170797043</v>
       </c>
-      <c r="F138" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A139" t="s">
+      <c r="D138" s="0"/>
+      <c r="E138" s="0"/>
+      <c r="F138" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G138" s="0"/>
+      <c r="H138" s="0"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="0" t="s">
         <v>448</v>
       </c>
-      <c r="B139" t="s">
+      <c r="B139" s="0" t="s">
         <v>450</v>
       </c>
-      <c r="C139">
+      <c r="C139" s="0">
         <v>5</v>
       </c>
-      <c r="F139" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A140" t="s">
+      <c r="D139" s="0"/>
+      <c r="E139" s="0"/>
+      <c r="F139" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G139" s="0"/>
+      <c r="H139" s="0"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="0" t="s">
         <v>449</v>
       </c>
-      <c r="B140" t="s">
+      <c r="B140" s="0" t="s">
         <v>450</v>
       </c>
-      <c r="C140">
+      <c r="C140" s="0">
         <v>-0.18284158980285484</v>
       </c>
-      <c r="F140" t="s">
-        <v>375</v>
-      </c>
+      <c r="D140" s="0"/>
+      <c r="E140" s="0"/>
+      <c r="F140" s="0" t="s">
+        <v>375</v>
+      </c>
+      <c r="G140" s="0"/>
+      <c r="H140" s="0"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>